<commit_message>
feat: add audit functionality and improve data import logic
</commit_message>
<xml_diff>
--- a/_VN30_AutoScore_PRO.xlsx
+++ b/_VN30_AutoScore_PRO.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DataVNF\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\dev\marketlens\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1651D31D-3CA6-4B12-8B47-45B6F14F542F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25287E7B-BD8A-475F-BD8F-F7636E1619B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13695" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13695" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Raw_VN30_Statistic" sheetId="1" r:id="rId1"/>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="255">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="333" uniqueCount="255">
   <si>
     <t>No.</t>
   </si>
@@ -847,7 +847,7 @@
     <numFmt numFmtId="166" formatCode="yyyy\-mm\-dd"/>
     <numFmt numFmtId="167" formatCode="h:mm;@"/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -915,14 +915,6 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -971,12 +963,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -1070,15 +1061,8 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="2" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="3">
-    <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
@@ -2106,7 +2090,7 @@
       <c r="B2" s="6">
         <v>46080</v>
       </c>
-      <c r="C2" s="48" t="s">
+      <c r="C2" t="s">
         <v>48</v>
       </c>
       <c r="D2" s="5">
@@ -2163,7 +2147,7 @@
       <c r="B3" s="6">
         <v>46080</v>
       </c>
-      <c r="C3" s="48" t="s">
+      <c r="C3" t="s">
         <v>51</v>
       </c>
       <c r="D3" s="5">
@@ -2220,7 +2204,7 @@
       <c r="B4" s="6">
         <v>46080</v>
       </c>
-      <c r="C4" s="48" t="s">
+      <c r="C4" t="s">
         <v>54</v>
       </c>
       <c r="D4" s="5">
@@ -2277,7 +2261,7 @@
       <c r="B5" s="6">
         <v>46080</v>
       </c>
-      <c r="C5" s="48" t="s">
+      <c r="C5" t="s">
         <v>70</v>
       </c>
       <c r="D5" s="5">
@@ -2334,7 +2318,7 @@
       <c r="B6" s="6">
         <v>46080</v>
       </c>
-      <c r="C6" s="48" t="s">
+      <c r="C6" t="s">
         <v>58</v>
       </c>
       <c r="D6" s="5">
@@ -2391,7 +2375,7 @@
       <c r="B7" s="6">
         <v>46080</v>
       </c>
-      <c r="C7" s="48" t="s">
+      <c r="C7" t="s">
         <v>60</v>
       </c>
       <c r="D7" s="5">
@@ -2448,7 +2432,7 @@
       <c r="B8" s="6">
         <v>46080</v>
       </c>
-      <c r="C8" s="48" t="s">
+      <c r="C8" t="s">
         <v>71</v>
       </c>
       <c r="D8" s="5">
@@ -2505,7 +2489,7 @@
       <c r="B9" s="6">
         <v>46080</v>
       </c>
-      <c r="C9" s="48" t="s">
+      <c r="C9" t="s">
         <v>56</v>
       </c>
       <c r="D9" s="5">
@@ -2562,7 +2546,7 @@
       <c r="B10" s="6">
         <v>46080</v>
       </c>
-      <c r="C10" s="48" t="s">
+      <c r="C10" t="s">
         <v>72</v>
       </c>
       <c r="D10" s="5">
@@ -2619,7 +2603,7 @@
       <c r="B11" s="6">
         <v>46080</v>
       </c>
-      <c r="C11" s="48" t="s">
+      <c r="C11" t="s">
         <v>57</v>
       </c>
       <c r="D11" s="5">
@@ -2676,7 +2660,7 @@
       <c r="B12" s="6">
         <v>46080</v>
       </c>
-      <c r="C12" s="48" t="s">
+      <c r="C12" t="s">
         <v>59</v>
       </c>
       <c r="D12" s="5">
@@ -2733,7 +2717,7 @@
       <c r="B13" s="6">
         <v>46080</v>
       </c>
-      <c r="C13" s="48" t="s">
+      <c r="C13" t="s">
         <v>73</v>
       </c>
       <c r="D13" s="5">
@@ -2790,7 +2774,7 @@
       <c r="B14" s="6">
         <v>46080</v>
       </c>
-      <c r="C14" s="48" t="s">
+      <c r="C14" t="s">
         <v>67</v>
       </c>
       <c r="D14" s="5">
@@ -2847,7 +2831,7 @@
       <c r="B15" s="6">
         <v>46080</v>
       </c>
-      <c r="C15" s="48" t="s">
+      <c r="C15" t="s">
         <v>74</v>
       </c>
       <c r="D15" s="5">
@@ -2904,7 +2888,7 @@
       <c r="B16" s="6">
         <v>46080</v>
       </c>
-      <c r="C16" s="48" t="s">
+      <c r="C16" t="s">
         <v>75</v>
       </c>
       <c r="D16" s="5">
@@ -2961,7 +2945,7 @@
       <c r="B17" s="6">
         <v>46080</v>
       </c>
-      <c r="C17" s="48" t="s">
+      <c r="C17" t="s">
         <v>61</v>
       </c>
       <c r="D17" s="5">
@@ -3018,7 +3002,7 @@
       <c r="B18" s="6">
         <v>46080</v>
       </c>
-      <c r="C18" s="48" t="s">
+      <c r="C18" t="s">
         <v>62</v>
       </c>
       <c r="D18" s="5">
@@ -3075,7 +3059,7 @@
       <c r="B19" s="6">
         <v>46080</v>
       </c>
-      <c r="C19" s="48" t="s">
+      <c r="C19" t="s">
         <v>76</v>
       </c>
       <c r="D19" s="5">
@@ -3132,7 +3116,7 @@
       <c r="B20" s="6">
         <v>46080</v>
       </c>
-      <c r="C20" s="48" t="s">
+      <c r="C20" t="s">
         <v>64</v>
       </c>
       <c r="D20" s="5">
@@ -3189,7 +3173,7 @@
       <c r="B21" s="6">
         <v>46080</v>
       </c>
-      <c r="C21" s="48" t="s">
+      <c r="C21" t="s">
         <v>66</v>
       </c>
       <c r="D21" s="5">
@@ -3246,7 +3230,7 @@
       <c r="B22" s="6">
         <v>46080</v>
       </c>
-      <c r="C22" s="48" t="s">
+      <c r="C22" t="s">
         <v>68</v>
       </c>
       <c r="D22" s="5">
@@ -3303,7 +3287,7 @@
       <c r="B23" s="6">
         <v>46080</v>
       </c>
-      <c r="C23" s="48" t="s">
+      <c r="C23" t="s">
         <v>55</v>
       </c>
       <c r="D23" s="5">
@@ -3360,7 +3344,7 @@
       <c r="B24" s="6">
         <v>46080</v>
       </c>
-      <c r="C24" s="48" t="s">
+      <c r="C24" t="s">
         <v>52</v>
       </c>
       <c r="D24" s="5">
@@ -3417,7 +3401,7 @@
       <c r="B25" s="6">
         <v>46080</v>
       </c>
-      <c r="C25" s="48" t="s">
+      <c r="C25" t="s">
         <v>69</v>
       </c>
       <c r="D25" s="5">
@@ -3474,7 +3458,7 @@
       <c r="B26" s="6">
         <v>46080</v>
       </c>
-      <c r="C26" s="48" t="s">
+      <c r="C26" t="s">
         <v>49</v>
       </c>
       <c r="D26" s="5">
@@ -3531,7 +3515,7 @@
       <c r="B27" s="6">
         <v>46080</v>
       </c>
-      <c r="C27" s="48" t="s">
+      <c r="C27" t="s">
         <v>77</v>
       </c>
       <c r="D27" s="5">
@@ -3588,7 +3572,7 @@
       <c r="B28" s="6">
         <v>46080</v>
       </c>
-      <c r="C28" s="48" t="s">
+      <c r="C28" t="s">
         <v>65</v>
       </c>
       <c r="D28" s="5">
@@ -3645,7 +3629,7 @@
       <c r="B29" s="6">
         <v>46080</v>
       </c>
-      <c r="C29" s="48" t="s">
+      <c r="C29" t="s">
         <v>63</v>
       </c>
       <c r="D29" s="5">
@@ -3702,7 +3686,7 @@
       <c r="B30" s="6">
         <v>46080</v>
       </c>
-      <c r="C30" s="48" t="s">
+      <c r="C30" t="s">
         <v>78</v>
       </c>
       <c r="D30" s="5">
@@ -3759,7 +3743,7 @@
       <c r="B31" s="6">
         <v>46080</v>
       </c>
-      <c r="C31" s="48" t="s">
+      <c r="C31" t="s">
         <v>79</v>
       </c>
       <c r="D31" s="5">
@@ -3810,45 +3794,13 @@
       <c r="S31" s="7"/>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="C2" r:id="rId1" tooltip="Asia Commercial Joint Stock Bank" display="https://finance.vietstock.vn/ACB-asia-commercial-joint-stock-bank.htm" xr:uid="{BF1FA7BD-02A2-48C4-8608-C4BE918EF1F8}"/>
-    <hyperlink ref="C3" r:id="rId2" tooltip="Joint Stock Commercial Bank for Investment and Development of Vietnam" display="https://finance.vietstock.vn/BID-joint-stock-commercial-bank-for-investment-and-development-of-vietnam.htm" xr:uid="{D7B58D66-5C07-4340-B045-D1F49AF21D8A}"/>
-    <hyperlink ref="C4" r:id="rId3" tooltip="Vietnam Joint Stock Commercial Bank For Industry And Trade" display="https://finance.vietstock.vn/CTG-vietnam-joint-stock-commercial-bank-for-industry-and-trade.htm" xr:uid="{1CE86BC0-01D9-4864-8DE5-BA30447D7BE6}"/>
-    <hyperlink ref="C5" r:id="rId4" tooltip="DucGiang Chemicals Group Joint Stock Company" display="https://finance.vietstock.vn/DGC-ducgiang-chemicals-group-joint-stock-company.htm" xr:uid="{E729336C-BD20-4AD4-B8C7-B00567918565}"/>
-    <hyperlink ref="C6" r:id="rId5" tooltip="FPT Corporation" display="https://finance.vietstock.vn/FPT-fpt-corporation.htm" xr:uid="{FC3327F6-F00C-43CB-825E-24619A19D67C}"/>
-    <hyperlink ref="C7" r:id="rId6" tooltip="PetroVietnam Gas Joint Stock Corporation" display="https://finance.vietstock.vn/GAS-petrovietnam-gas-joint-stock-corporation.htm" xr:uid="{0161297D-5913-4813-A222-B9D7A8BBA205}"/>
-    <hyperlink ref="C8" r:id="rId7" tooltip="Viet Nam Rubber Group - Joint Stock Company" display="https://finance.vietstock.vn/GVR-viet-nam-rubber-group-joint-stock-company.htm" xr:uid="{2EDB68B8-2B08-44D3-BFFD-C0C692654365}"/>
-    <hyperlink ref="C9" r:id="rId8" tooltip="Ho Chi Minh City Development Joint Stock Commercial Bank" display="https://finance.vietstock.vn/HDB-ho-chi-minh-city-development-joint-stock-commercial-bank.htm" xr:uid="{D3D4D6BB-012A-4B1A-90FD-7625BA4F5F7B}"/>
-    <hyperlink ref="C10" r:id="rId9" tooltip="Hoa Phat Group Joint Stock Company" display="https://finance.vietstock.vn/HPG-hoa-phat-group-joint-stock-company.htm" xr:uid="{FA15FA95-53B6-4A98-A871-B0F523EA27F2}"/>
-    <hyperlink ref="C11" r:id="rId10" tooltip="Fortune Vietnam Joint Stock Commercial Bank" display="https://finance.vietstock.vn/LPB-fortune-vietnam-joint-stock-commercial-bank.htm" xr:uid="{E920BDBF-7EA1-4EF0-AEF0-E66D608B32F3}"/>
-    <hyperlink ref="C12" r:id="rId11" tooltip="Military Commercial Joint Stock Bank" display="https://finance.vietstock.vn/MBB-military-commercial-joint-stock-bank.htm" xr:uid="{29698533-3D24-4104-BBAE-1F2FB8BC6B36}"/>
-    <hyperlink ref="C13" r:id="rId12" tooltip="Masan Group Corporation" display="https://finance.vietstock.vn/MSN-masan-group-corporation.htm" xr:uid="{96375D59-965E-477F-BEA1-85195A490AAF}"/>
-    <hyperlink ref="C14" r:id="rId13" tooltip="Mobile World Investment Corporation" display="https://finance.vietstock.vn/MWG-mobile-world-investment-corporation.htm" xr:uid="{98872C06-9FF4-40FA-8476-8CCE88D0D223}"/>
-    <hyperlink ref="C15" r:id="rId14" tooltip="VietNam National Petroleum Group" display="https://finance.vietstock.vn/PLX-vietnam-national-petroleum-group.htm" xr:uid="{A360E07B-3DD5-41BB-B089-1C1D1815DB11}"/>
-    <hyperlink ref="C16" r:id="rId15" tooltip="Saigon Beer - Alcohol - Beverage Corporation" display="https://finance.vietstock.vn/SAB-saigon-beer-alcohol-beverage-corporation.htm" xr:uid="{F0BAE27C-49CC-46CC-AB87-B925D1DA0E99}"/>
-    <hyperlink ref="C17" r:id="rId16" tooltip="Saigon Hanoi Commercial Joint Stock Bank" display="https://finance.vietstock.vn/SHB-saigon-hanoi-commercial-joint-stock-bank.htm" xr:uid="{401271DF-F15C-42D4-9BB1-904ED32D0FF1}"/>
-    <hyperlink ref="C18" r:id="rId17" tooltip="Southeast Asia Commercial Joint Stock Bank" display="https://finance.vietstock.vn/SSB-southeast-asia-commercial-joint-stock-bank.htm" xr:uid="{BE92D4B4-7E7B-4F01-BEC8-EAB28D645909}"/>
-    <hyperlink ref="C19" r:id="rId18" tooltip="SSI Securities Corporation" display="https://finance.vietstock.vn/SSI-ssi-securities-corporation.htm" xr:uid="{B5C87DE3-EF3E-4B7B-ABC9-4BD5335B90E5}"/>
-    <hyperlink ref="C20" r:id="rId19" tooltip="Saigon Thuong Tin Commercial Joint Stock Bank" display="https://finance.vietstock.vn/STB-saigon-thuong-tin-commercial-joint-stock-bank.htm" xr:uid="{EE352CF9-3A4A-47A4-89F9-1C22E4E0FD92}"/>
-    <hyperlink ref="C21" r:id="rId20" tooltip="Vietnam Technological and Commercial Joint Stock Bank" display="https://finance.vietstock.vn/TCB-vietnam-technological-and-commercial-joint-stock-bank.htm" xr:uid="{CF47D3C2-99E9-464A-8A04-764516CCA170}"/>
-    <hyperlink ref="C22" r:id="rId21" tooltip="Tien Phong Commercial Joint Stock Bank" display="https://finance.vietstock.vn/TPB-tien-phong-commercial-joint-stock-bank.htm" xr:uid="{8ADFEAFA-8226-487E-80A4-F67C55BEF120}"/>
-    <hyperlink ref="C23" r:id="rId22" tooltip="Joint Stock Commercial Bank for Foreign Trade of Vietnam" display="https://finance.vietstock.vn/VCB-joint-stock-commercial-bank-for-foreign-trade-of-vietnam.htm" xr:uid="{E1F04473-C0FA-4C0D-B297-FED64154F585}"/>
-    <hyperlink ref="C24" r:id="rId23" tooltip="Vinhomes Joint Stock Company" display="https://finance.vietstock.vn/VHM-vinhomes-joint-stock-company.htm" xr:uid="{AF83D29A-5000-4940-8EAA-9B60E0572E21}"/>
-    <hyperlink ref="C25" r:id="rId24" tooltip="Vietnam International Commercial Joint Stock Bank" display="https://finance.vietstock.vn/VIB-vietnam-international-commercial-joint-stock-bank.htm" xr:uid="{D826BB3F-C840-42E8-BADB-EBCD1B4F5E99}"/>
-    <hyperlink ref="C26" r:id="rId25" tooltip="Vingroup Joint Stock Company" display="https://finance.vietstock.vn/VIC-vingroup-joint-stock-company.htm" xr:uid="{0F183890-919A-4F2B-9F7E-8908B78FB076}"/>
-    <hyperlink ref="C27" r:id="rId26" tooltip="Vietjet Aviation Joint Stock Company" display="https://finance.vietstock.vn/VJC-vietjet-aviation-joint-stock-company.htm" xr:uid="{87654CEA-863D-4C68-A530-BD60F94A651B}"/>
-    <hyperlink ref="C28" r:id="rId27" tooltip="Vietnam Dairy Products Joint Stock Company" display="https://finance.vietstock.vn/VNM-vietnam-dairy-products-joint-stock-company.htm" xr:uid="{6EE93E8E-8ECD-4D29-8BF8-03963881A862}"/>
-    <hyperlink ref="C29" r:id="rId28" tooltip="Vietnam Prosperity Joint Stock Commercial Bank" display="https://finance.vietstock.vn/VPB-vietnam-prosperity-joint-stock-commercial-bank.htm" xr:uid="{A4A97E97-81AC-4873-A6A3-80CAA54B9852}"/>
-    <hyperlink ref="C30" r:id="rId29" tooltip="Vinpearl Joint Stock Company" display="https://finance.vietstock.vn/VPL-vinpearl-joint-stock-company.htm" xr:uid="{38390046-EC96-4F90-B0ED-A13926026DAF}"/>
-    <hyperlink ref="C31" r:id="rId30" tooltip="Vincom Retail Joint Stock Company" display="https://finance.vietstock.vn/VRE-vincom-retail-joint-stock-company.htm" xr:uid="{6A4E7F8D-4894-4978-A8EA-61DD282EA566}"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{07B554F5-542D-41F2-AA0F-AF2746E845A9}">
-  <dimension ref="A1:I32"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="3" max="3" width="14.53125" customWidth="1"/>
@@ -3890,937 +3842,876 @@
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A2" s="30" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="30" t="s">
-        <v>115</v>
-      </c>
-      <c r="C2" s="30" t="s">
-        <v>19</v>
-      </c>
-      <c r="D2" s="30" t="s">
-        <v>116</v>
-      </c>
-      <c r="E2" s="30" t="s">
-        <v>117</v>
-      </c>
-      <c r="F2" s="30" t="s">
-        <v>16</v>
-      </c>
-      <c r="G2" s="30" t="s">
-        <v>118</v>
-      </c>
-      <c r="H2" s="30" t="s">
-        <v>119</v>
-      </c>
-      <c r="I2" s="30" t="s">
-        <v>120</v>
+      <c r="A2" s="5">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C2" s="7">
+        <v>92900</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>230</v>
+      </c>
+      <c r="E2" s="7">
+        <v>1703507121</v>
+      </c>
+      <c r="F2" s="7">
+        <v>118725092376099</v>
+      </c>
+      <c r="G2" s="5">
+        <v>8.9718999999999998</v>
+      </c>
+      <c r="H2" s="5">
+        <v>0.23780000000000001</v>
+      </c>
+      <c r="I2" s="5">
+        <v>4.9211</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A3" s="5">
-        <v>1</v>
-      </c>
-      <c r="B3" s="48" t="s">
-        <v>58</v>
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>49</v>
       </c>
       <c r="C3" s="7">
-        <v>92900</v>
+        <v>172000</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="E3" s="7">
-        <v>1703507121</v>
+        <v>7706031024</v>
       </c>
       <c r="F3" s="7">
-        <v>118725092376099</v>
+        <v>142139899926367</v>
       </c>
       <c r="G3" s="5">
-        <v>8.9718999999999998</v>
+        <v>10.741300000000001</v>
       </c>
       <c r="H3" s="5">
-        <v>0.23780000000000001</v>
+        <v>0.1976</v>
       </c>
       <c r="I3" s="5">
-        <v>4.9211</v>
+        <v>4.0907999999999998</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A4" s="5">
-        <v>2</v>
-      </c>
-      <c r="B4" s="48" t="s">
-        <v>49</v>
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>60</v>
       </c>
       <c r="C4" s="7">
-        <v>172000</v>
+        <v>107900</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="E4" s="7">
-        <v>7706031024</v>
+        <v>2412949756</v>
       </c>
       <c r="F4" s="7">
-        <v>142139899926367</v>
+        <v>13017863933620</v>
       </c>
       <c r="G4" s="5">
-        <v>10.741300000000001</v>
+        <v>0.98370000000000002</v>
       </c>
       <c r="H4" s="5">
-        <v>0.1976</v>
+        <v>1.7600000000000001E-2</v>
       </c>
       <c r="I4" s="5">
-        <v>4.0907999999999998</v>
+        <v>0.36449999999999999</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A5" s="5">
-        <v>3</v>
-      </c>
-      <c r="B5" s="48" t="s">
-        <v>60</v>
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>48</v>
       </c>
       <c r="C5" s="7">
-        <v>107900</v>
+        <v>24550</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>232</v>
+        <v>222</v>
       </c>
       <c r="E5" s="7">
-        <v>2412949756</v>
+        <v>5136656599</v>
       </c>
       <c r="F5" s="7">
-        <v>13017863933620</v>
+        <v>48513823582942</v>
       </c>
       <c r="G5" s="5">
-        <v>0.98370000000000002</v>
+        <v>3.6661000000000001</v>
       </c>
       <c r="H5" s="5">
-        <v>1.7600000000000001E-2</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="I5" s="5">
-        <v>0.36449999999999999</v>
+        <v>0.31109999999999999</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A6" s="5">
-        <v>4</v>
-      </c>
-      <c r="B6" s="48" t="s">
-        <v>48</v>
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>78</v>
       </c>
       <c r="C6" s="7">
-        <v>24550</v>
+        <v>83500</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>222</v>
+        <v>233</v>
       </c>
       <c r="E6" s="7">
-        <v>5136656599</v>
+        <v>1793300377</v>
       </c>
       <c r="F6" s="7">
-        <v>48513823582942</v>
+        <v>8479060426277</v>
       </c>
       <c r="G6" s="5">
-        <v>3.6661000000000001</v>
+        <v>0.64070000000000005</v>
       </c>
       <c r="H6" s="5">
-        <v>1.4999999999999999E-2</v>
+        <v>1.41E-2</v>
       </c>
       <c r="I6" s="5">
-        <v>0.31109999999999999</v>
+        <v>0.29170000000000001</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A7" s="5">
-        <v>5</v>
-      </c>
-      <c r="B7" s="48" t="s">
-        <v>78</v>
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>52</v>
       </c>
       <c r="C7" s="7">
-        <v>83500</v>
+        <v>108000</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="E7" s="7">
-        <v>1793300377</v>
+        <v>4107412004</v>
       </c>
       <c r="F7" s="7">
-        <v>8479060426277</v>
+        <v>50237756220924</v>
       </c>
       <c r="G7" s="5">
-        <v>0.64070000000000005</v>
+        <v>3.7964000000000002</v>
       </c>
       <c r="H7" s="5">
-        <v>1.41E-2</v>
+        <v>1.4E-2</v>
       </c>
       <c r="I7" s="5">
-        <v>0.29170000000000001</v>
+        <v>0.29070000000000001</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A8" s="5">
-        <v>6</v>
-      </c>
-      <c r="B8" s="48" t="s">
-        <v>52</v>
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>63</v>
       </c>
       <c r="C8" s="7">
-        <v>108000</v>
+        <v>28950</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>234</v>
+        <v>224</v>
       </c>
       <c r="E8" s="7">
-        <v>4107412004</v>
+        <v>7933923601</v>
       </c>
       <c r="F8" s="7">
-        <v>50237756220924</v>
+        <v>62373825684885</v>
       </c>
       <c r="G8" s="5">
-        <v>3.7964000000000002</v>
+        <v>4.7134999999999998</v>
       </c>
       <c r="H8" s="5">
-        <v>1.4E-2</v>
+        <v>8.0000000000000002E-3</v>
       </c>
       <c r="I8" s="5">
-        <v>0.29070000000000001</v>
+        <v>0.16589999999999999</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A9" s="5">
-        <v>7</v>
-      </c>
-      <c r="B9" s="48" t="s">
-        <v>63</v>
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>70</v>
       </c>
       <c r="C9" s="7">
-        <v>28950</v>
+        <v>73800</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>224</v>
+        <v>235</v>
       </c>
       <c r="E9" s="7">
-        <v>7933923601</v>
+        <v>379778413</v>
       </c>
       <c r="F9" s="7">
-        <v>62373825684885</v>
+        <v>16816588127640</v>
       </c>
       <c r="G9" s="5">
-        <v>4.7134999999999998</v>
+        <v>1.2707999999999999</v>
       </c>
       <c r="H9" s="5">
-        <v>8.0000000000000002E-3</v>
+        <v>3.3999999999999998E-3</v>
       </c>
       <c r="I9" s="5">
-        <v>0.16589999999999999</v>
+        <v>7.0999999999999994E-2</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A10" s="5">
-        <v>8</v>
-      </c>
-      <c r="B10" s="48" t="s">
-        <v>70</v>
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>74</v>
       </c>
       <c r="C10" s="7">
-        <v>73800</v>
+        <v>57800</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>235</v>
+        <v>211</v>
       </c>
       <c r="E10" s="7">
-        <v>379778413</v>
+        <v>1270592235</v>
       </c>
       <c r="F10" s="7">
-        <v>16816588127640</v>
+        <v>7344023118300</v>
       </c>
       <c r="G10" s="5">
-        <v>1.2707999999999999</v>
+        <v>0.55489999999999995</v>
       </c>
       <c r="H10" s="5">
-        <v>3.3999999999999998E-3</v>
+        <v>2.8999999999999998E-3</v>
       </c>
       <c r="I10" s="5">
-        <v>7.0999999999999994E-2</v>
+        <v>5.9700000000000003E-2</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A11" s="5">
-        <v>9</v>
-      </c>
-      <c r="B11" s="48" t="s">
-        <v>74</v>
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>68</v>
       </c>
       <c r="C11" s="7">
-        <v>57800</v>
+        <v>18400</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>211</v>
+        <v>236</v>
       </c>
       <c r="E11" s="7">
-        <v>1270592235</v>
+        <v>2774046873</v>
       </c>
       <c r="F11" s="7">
-        <v>7344023118300</v>
+        <v>12706000180964</v>
       </c>
       <c r="G11" s="5">
-        <v>0.55489999999999995</v>
+        <v>0.96009999999999995</v>
       </c>
       <c r="H11" s="5">
-        <v>2.8999999999999998E-3</v>
+        <v>2.5999999999999999E-3</v>
       </c>
       <c r="I11" s="5">
-        <v>5.9700000000000003E-2</v>
+        <v>5.3699999999999998E-2</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A12" s="5">
-        <v>10</v>
-      </c>
-      <c r="B12" s="48" t="s">
-        <v>68</v>
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>76</v>
       </c>
       <c r="C12" s="7">
-        <v>18400</v>
+        <v>32400</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>236</v>
+        <v>223</v>
       </c>
       <c r="E12" s="7">
-        <v>2774046873</v>
+        <v>2491097752</v>
       </c>
       <c r="F12" s="7">
-        <v>12706000180964</v>
+        <v>25571038709152</v>
       </c>
       <c r="G12" s="5">
-        <v>0.96009999999999995</v>
+        <v>1.9322999999999999</v>
       </c>
       <c r="H12" s="5">
-        <v>2.5999999999999999E-3</v>
+        <v>0</v>
       </c>
       <c r="I12" s="5">
-        <v>5.3699999999999998E-2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A13" s="5">
-        <v>11</v>
-      </c>
-      <c r="B13" s="48" t="s">
-        <v>76</v>
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>62</v>
       </c>
       <c r="C13" s="7">
-        <v>32400</v>
+        <v>16900</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>223</v>
+        <v>237</v>
       </c>
       <c r="E13" s="7">
-        <v>2491097752</v>
+        <v>2845000000</v>
       </c>
       <c r="F13" s="7">
-        <v>25571038709152</v>
+        <v>10880617150000</v>
       </c>
       <c r="G13" s="5">
-        <v>1.9322999999999999</v>
+        <v>0.82220000000000004</v>
       </c>
       <c r="H13" s="5">
-        <v>0</v>
+        <v>-4.8999999999999998E-3</v>
       </c>
       <c r="I13" s="5">
-        <v>0</v>
+        <v>-0.1004</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A14" s="5">
-        <v>12</v>
-      </c>
-      <c r="B14" s="48" t="s">
-        <v>62</v>
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>51</v>
       </c>
       <c r="C14" s="7">
-        <v>16900</v>
+        <v>47900</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="E14" s="7">
-        <v>2845000000</v>
+        <v>7021361917</v>
       </c>
       <c r="F14" s="7">
-        <v>10880617150000</v>
+        <v>6088795861363</v>
       </c>
       <c r="G14" s="5">
-        <v>0.82220000000000004</v>
+        <v>0.46010000000000001</v>
       </c>
       <c r="H14" s="5">
-        <v>-4.8999999999999998E-3</v>
+        <v>-5.1999999999999998E-3</v>
       </c>
       <c r="I14" s="5">
-        <v>-0.1004</v>
+        <v>-0.1086</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A15" s="5">
-        <v>13</v>
-      </c>
-      <c r="B15" s="48" t="s">
-        <v>51</v>
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>75</v>
       </c>
       <c r="C15" s="7">
-        <v>47900</v>
+        <v>48400</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="E15" s="7">
-        <v>7021361917</v>
+        <v>1282562372</v>
       </c>
       <c r="F15" s="7">
-        <v>6088795861363</v>
+        <v>6828362068528</v>
       </c>
       <c r="G15" s="5">
-        <v>0.46010000000000001</v>
+        <v>0.51600000000000001</v>
       </c>
       <c r="H15" s="5">
-        <v>-5.1999999999999998E-3</v>
+        <v>-7.4000000000000003E-3</v>
       </c>
       <c r="I15" s="5">
-        <v>-0.1086</v>
+        <v>-0.1527</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A16" s="5">
-        <v>14</v>
-      </c>
-      <c r="B16" s="48" t="s">
-        <v>75</v>
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>69</v>
       </c>
       <c r="C16" s="7">
-        <v>48400</v>
+        <v>17300</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="E16" s="7">
-        <v>1282562372</v>
+        <v>3404005710</v>
       </c>
       <c r="F16" s="7">
-        <v>6828362068528</v>
+        <v>17324642808971</v>
       </c>
       <c r="G16" s="5">
-        <v>0.51600000000000001</v>
+        <v>1.3091999999999999</v>
       </c>
       <c r="H16" s="5">
-        <v>-7.4000000000000003E-3</v>
+        <v>-7.4999999999999997E-3</v>
       </c>
       <c r="I16" s="5">
-        <v>-0.1527</v>
+        <v>-0.1545</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A17" s="5">
-        <v>15</v>
-      </c>
-      <c r="B17" s="48" t="s">
-        <v>69</v>
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>71</v>
       </c>
       <c r="C17" s="7">
-        <v>17300</v>
+        <v>40000</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="E17" s="7">
-        <v>3404005710</v>
+        <v>4000000000</v>
       </c>
       <c r="F17" s="7">
-        <v>17324642808971</v>
+        <v>6400000000000</v>
       </c>
       <c r="G17" s="5">
-        <v>1.3091999999999999</v>
+        <v>0.48359999999999997</v>
       </c>
       <c r="H17" s="5">
-        <v>-7.4999999999999997E-3</v>
+        <v>-9.4999999999999998E-3</v>
       </c>
       <c r="I17" s="5">
-        <v>-0.1545</v>
+        <v>-0.19620000000000001</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A18" s="5">
-        <v>16</v>
-      </c>
-      <c r="B18" s="48" t="s">
-        <v>71</v>
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>57</v>
       </c>
       <c r="C18" s="7">
-        <v>40000</v>
+        <v>43050</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="E18" s="7">
-        <v>4000000000</v>
+        <v>2987282100</v>
       </c>
       <c r="F18" s="7">
-        <v>6400000000000</v>
+        <v>55295214519318</v>
       </c>
       <c r="G18" s="5">
-        <v>0.48359999999999997</v>
+        <v>4.1784999999999997</v>
       </c>
       <c r="H18" s="5">
-        <v>-9.4999999999999998E-3</v>
+        <v>-9.5999999999999992E-3</v>
       </c>
       <c r="I18" s="5">
-        <v>-0.19620000000000001</v>
+        <v>-0.19889999999999999</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A19" s="5">
-        <v>17</v>
-      </c>
-      <c r="B19" s="48" t="s">
-        <v>57</v>
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>54</v>
       </c>
       <c r="C19" s="7">
-        <v>43050</v>
+        <v>38250</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="E19" s="7">
-        <v>2987282100</v>
+        <v>7766944637</v>
       </c>
       <c r="F19" s="7">
-        <v>55295214519318</v>
+        <v>20169143581277</v>
       </c>
       <c r="G19" s="5">
-        <v>4.1784999999999997</v>
+        <v>1.5241</v>
       </c>
       <c r="H19" s="5">
-        <v>-9.5999999999999992E-3</v>
+        <v>-9.9000000000000008E-3</v>
       </c>
       <c r="I19" s="5">
-        <v>-0.19889999999999999</v>
+        <v>-0.20499999999999999</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A20" s="5">
-        <v>18</v>
-      </c>
-      <c r="B20" s="48" t="s">
-        <v>54</v>
+        <v>19</v>
+      </c>
+      <c r="B20" t="s">
+        <v>55</v>
       </c>
       <c r="C20" s="7">
-        <v>38250</v>
+        <v>64900</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="E20" s="7">
-        <v>7766944637</v>
+        <v>8355675094</v>
       </c>
       <c r="F20" s="7">
-        <v>20169143581277</v>
+        <v>26998117050919</v>
       </c>
       <c r="G20" s="5">
-        <v>1.5241</v>
+        <v>2.0402</v>
       </c>
       <c r="H20" s="5">
-        <v>-9.9000000000000008E-3</v>
+        <v>-1.55E-2</v>
       </c>
       <c r="I20" s="5">
-        <v>-0.20499999999999999</v>
+        <v>-0.32090000000000002</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A21" s="5">
-        <v>19</v>
-      </c>
-      <c r="B21" s="48" t="s">
-        <v>55</v>
+        <v>20</v>
+      </c>
+      <c r="B21" t="s">
+        <v>61</v>
       </c>
       <c r="C21" s="7">
-        <v>64900</v>
+        <v>15950</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="E21" s="7">
-        <v>8355675094</v>
+        <v>4593703838</v>
       </c>
       <c r="F21" s="7">
-        <v>26998117050919</v>
+        <v>24871357646555</v>
       </c>
       <c r="G21" s="5">
-        <v>2.0402</v>
+        <v>1.8794999999999999</v>
       </c>
       <c r="H21" s="5">
-        <v>-1.55E-2</v>
+        <v>-2.3300000000000001E-2</v>
       </c>
       <c r="I21" s="5">
-        <v>-0.32090000000000002</v>
+        <v>-0.4824</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A22" s="5">
-        <v>20</v>
-      </c>
-      <c r="B22" s="48" t="s">
-        <v>61</v>
+        <v>21</v>
+      </c>
+      <c r="B22" t="s">
+        <v>66</v>
       </c>
       <c r="C22" s="7">
-        <v>15950</v>
+        <v>36250</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="E22" s="7">
-        <v>4593703838</v>
+        <v>7086240414</v>
       </c>
       <c r="F22" s="7">
-        <v>24871357646555</v>
+        <v>63944196201817</v>
       </c>
       <c r="G22" s="5">
-        <v>1.8794999999999999</v>
+        <v>4.8320999999999996</v>
       </c>
       <c r="H22" s="5">
-        <v>-2.3300000000000001E-2</v>
+        <v>-2.6599999999999999E-2</v>
       </c>
       <c r="I22" s="5">
-        <v>-0.4824</v>
+        <v>-0.55010000000000003</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A23" s="5">
-        <v>21</v>
-      </c>
-      <c r="B23" s="48" t="s">
-        <v>66</v>
+        <v>22</v>
+      </c>
+      <c r="B23" t="s">
+        <v>59</v>
       </c>
       <c r="C23" s="7">
-        <v>36250</v>
+        <v>28500</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="E23" s="7">
-        <v>7086240414</v>
+        <v>8054999909</v>
       </c>
       <c r="F23" s="7">
-        <v>63944196201817</v>
+        <v>51951124663091</v>
       </c>
       <c r="G23" s="5">
-        <v>4.8320999999999996</v>
+        <v>3.9258000000000002</v>
       </c>
       <c r="H23" s="5">
-        <v>-2.6599999999999999E-2</v>
+        <v>-4.0800000000000003E-2</v>
       </c>
       <c r="I23" s="5">
-        <v>-0.55010000000000003</v>
+        <v>-0.84509999999999996</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A24" s="5">
-        <v>22</v>
-      </c>
-      <c r="B24" s="48" t="s">
-        <v>59</v>
+        <v>23</v>
+      </c>
+      <c r="B24" t="s">
+        <v>67</v>
       </c>
       <c r="C24" s="7">
-        <v>28500</v>
+        <v>93100</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="E24" s="7">
-        <v>8054999909</v>
+        <v>1468456763</v>
       </c>
       <c r="F24" s="7">
-        <v>51951124663091</v>
+        <v>102534993476475</v>
       </c>
       <c r="G24" s="5">
-        <v>3.9258000000000002</v>
+        <v>7.7484000000000002</v>
       </c>
       <c r="H24" s="5">
-        <v>-4.0800000000000003E-2</v>
+        <v>-4.1099999999999998E-2</v>
       </c>
       <c r="I24" s="5">
-        <v>-0.84509999999999996</v>
+        <v>-0.85</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A25" s="5">
-        <v>23</v>
-      </c>
-      <c r="B25" s="48" t="s">
-        <v>67</v>
+        <v>24</v>
+      </c>
+      <c r="B25" t="s">
+        <v>79</v>
       </c>
       <c r="C25" s="7">
-        <v>93100</v>
+        <v>29050</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="E25" s="7">
-        <v>1468456763</v>
+        <v>2272318410</v>
       </c>
       <c r="F25" s="7">
-        <v>102534993476475</v>
+        <v>26404339924200</v>
       </c>
       <c r="G25" s="5">
-        <v>7.7484000000000002</v>
+        <v>1.9953000000000001</v>
       </c>
       <c r="H25" s="5">
-        <v>-4.1099999999999998E-2</v>
+        <v>-4.6899999999999997E-2</v>
       </c>
       <c r="I25" s="5">
-        <v>-0.85</v>
+        <v>-0.97050000000000003</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A26" s="5">
-        <v>24</v>
-      </c>
-      <c r="B26" s="48" t="s">
-        <v>79</v>
+        <v>25</v>
+      </c>
+      <c r="B26" t="s">
+        <v>77</v>
       </c>
       <c r="C26" s="7">
-        <v>29050</v>
+        <v>175800</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="E26" s="7">
-        <v>2272318410</v>
+        <v>591611334</v>
       </c>
       <c r="F26" s="7">
-        <v>26404339924200</v>
+        <v>46802372632740</v>
       </c>
       <c r="G26" s="5">
-        <v>1.9953000000000001</v>
+        <v>3.5367999999999999</v>
       </c>
       <c r="H26" s="5">
-        <v>-4.6899999999999997E-2</v>
+        <v>-5.3400000000000003E-2</v>
       </c>
       <c r="I26" s="5">
-        <v>-0.97050000000000003</v>
+        <v>-1.1053999999999999</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A27" s="5">
-        <v>25</v>
-      </c>
-      <c r="B27" s="48" t="s">
-        <v>77</v>
+        <v>26</v>
+      </c>
+      <c r="B27" t="s">
+        <v>56</v>
       </c>
       <c r="C27" s="7">
-        <v>175800</v>
+        <v>27950</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>250</v>
+        <v>227</v>
       </c>
       <c r="E27" s="7">
-        <v>591611334</v>
+        <v>5005276323</v>
       </c>
       <c r="F27" s="7">
-        <v>46802372632740</v>
+        <v>50654077106340</v>
       </c>
       <c r="G27" s="5">
-        <v>3.5367999999999999</v>
+        <v>3.8277999999999999</v>
       </c>
       <c r="H27" s="5">
-        <v>-5.3400000000000003E-2</v>
+        <v>-6.0499999999999998E-2</v>
       </c>
       <c r="I27" s="5">
-        <v>-1.1053999999999999</v>
+        <v>-1.2518</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A28" s="5">
-        <v>26</v>
-      </c>
-      <c r="B28" s="48" t="s">
-        <v>56</v>
+        <v>27</v>
+      </c>
+      <c r="B28" t="s">
+        <v>64</v>
       </c>
       <c r="C28" s="7">
-        <v>27950</v>
+        <v>65500</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>227</v>
+        <v>251</v>
       </c>
       <c r="E28" s="7">
-        <v>5005276323</v>
+        <v>1885215716</v>
       </c>
       <c r="F28" s="7">
-        <v>50654077106340</v>
+        <v>53093396192258</v>
       </c>
       <c r="G28" s="5">
-        <v>3.8277999999999999</v>
+        <v>4.0122</v>
       </c>
       <c r="H28" s="5">
-        <v>-6.0499999999999998E-2</v>
+        <v>-8.9899999999999994E-2</v>
       </c>
       <c r="I28" s="5">
-        <v>-1.2518</v>
+        <v>-1.8602000000000001</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A29" s="5">
-        <v>27</v>
-      </c>
-      <c r="B29" s="48" t="s">
-        <v>64</v>
+        <v>28</v>
+      </c>
+      <c r="B29" t="s">
+        <v>73</v>
       </c>
       <c r="C29" s="7">
-        <v>65500</v>
+        <v>79000</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="E29" s="7">
-        <v>1885215716</v>
+        <v>1445915457</v>
       </c>
       <c r="F29" s="7">
-        <v>53093396192258</v>
+        <v>68536392661800</v>
       </c>
       <c r="G29" s="5">
-        <v>4.0122</v>
+        <v>5.1791999999999998</v>
       </c>
       <c r="H29" s="5">
-        <v>-8.9899999999999994E-2</v>
+        <v>-9.01E-2</v>
       </c>
       <c r="I29" s="5">
-        <v>-1.8602000000000001</v>
+        <v>-1.8653</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A30" s="5">
-        <v>28</v>
-      </c>
-      <c r="B30" s="48" t="s">
-        <v>73</v>
+        <v>29</v>
+      </c>
+      <c r="B30" t="s">
+        <v>65</v>
       </c>
       <c r="C30" s="7">
-        <v>79000</v>
+        <v>68200</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="E30" s="7">
-        <v>1445915457</v>
+        <v>2089955445</v>
       </c>
       <c r="F30" s="7">
-        <v>68536392661800</v>
+        <v>57013984539600</v>
       </c>
       <c r="G30" s="5">
-        <v>5.1791999999999998</v>
+        <v>4.3083999999999998</v>
       </c>
       <c r="H30" s="5">
-        <v>-9.01E-2</v>
+        <v>-0.14649999999999999</v>
       </c>
       <c r="I30" s="5">
-        <v>-1.8653</v>
+        <v>-3.032</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A31" s="5">
-        <v>29</v>
-      </c>
-      <c r="B31" s="48" t="s">
-        <v>65</v>
+        <v>30</v>
+      </c>
+      <c r="B31" t="s">
+        <v>72</v>
       </c>
       <c r="C31" s="7">
-        <v>68200</v>
+        <v>28800</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="E31" s="7">
-        <v>2089955445</v>
+        <v>7675465855</v>
       </c>
       <c r="F31" s="7">
-        <v>57013984539600</v>
+        <v>121579379143200</v>
       </c>
       <c r="G31" s="5">
-        <v>4.3083999999999998</v>
+        <v>9.1875999999999998</v>
       </c>
       <c r="H31" s="5">
-        <v>-0.14649999999999999</v>
+        <v>-0.18740000000000001</v>
       </c>
       <c r="I31" s="5">
-        <v>-3.032</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A32" s="5">
-        <v>30</v>
-      </c>
-      <c r="B32" s="48" t="s">
-        <v>72</v>
-      </c>
-      <c r="C32" s="7">
-        <v>28800</v>
-      </c>
-      <c r="D32" s="5" t="s">
-        <v>254</v>
-      </c>
-      <c r="E32" s="7">
-        <v>7675465855</v>
-      </c>
-      <c r="F32" s="7">
-        <v>121579379143200</v>
-      </c>
-      <c r="G32" s="5">
-        <v>9.1875999999999998</v>
-      </c>
-      <c r="H32" s="5">
-        <v>-0.18740000000000001</v>
-      </c>
-      <c r="I32" s="5">
         <v>-3.8794</v>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="B3" r:id="rId1" display="https://finance.vietstock.vn/FPT-fpt-corporation.htm" xr:uid="{AA991268-95FC-48C7-B885-EC599F8205FC}"/>
-    <hyperlink ref="B4" r:id="rId2" display="https://finance.vietstock.vn/VIC-vingroup-joint-stock-company.htm" xr:uid="{F2636971-F665-4F1F-87D9-D8BB0A2889D5}"/>
-    <hyperlink ref="B5" r:id="rId3" display="https://finance.vietstock.vn/GAS-petrovietnam-gas-joint-stock-corporation.htm" xr:uid="{95F4482F-D67B-44F0-945A-CFAC737063B3}"/>
-    <hyperlink ref="B6" r:id="rId4" display="https://finance.vietstock.vn/ACB-asia-commercial-joint-stock-bank.htm" xr:uid="{C5A4DF1B-2317-46B7-8593-667861A2FB65}"/>
-    <hyperlink ref="B7" r:id="rId5" display="https://finance.vietstock.vn/VPL-vinpearl-joint-stock-company.htm" xr:uid="{A3A7E5A3-7DB3-4DEE-BA34-E8032BFF2BF0}"/>
-    <hyperlink ref="B8" r:id="rId6" display="https://finance.vietstock.vn/VHM-vinhomes-joint-stock-company.htm" xr:uid="{22FE340C-5FD4-49B3-9921-D0584E433973}"/>
-    <hyperlink ref="B9" r:id="rId7" display="https://finance.vietstock.vn/VPB-vietnam-prosperity-joint-stock-commercial-bank.htm" xr:uid="{696B6971-C0C1-4D51-AB82-03656BD88B69}"/>
-    <hyperlink ref="B10" r:id="rId8" display="https://finance.vietstock.vn/DGC-ducgiang-chemicals-group-joint-stock-company.htm" xr:uid="{7457A1BB-8789-4BCD-A91F-9063504F3A47}"/>
-    <hyperlink ref="B11" r:id="rId9" display="https://finance.vietstock.vn/PLX-vietnam-national-petroleum-group.htm" xr:uid="{25152359-15DD-477E-9BED-3D0F7649A265}"/>
-    <hyperlink ref="B12" r:id="rId10" display="https://finance.vietstock.vn/TPB-tien-phong-commercial-joint-stock-bank.htm" xr:uid="{9182672E-23E2-4014-9D6F-872F3A0DB0D2}"/>
-    <hyperlink ref="B13" r:id="rId11" display="https://finance.vietstock.vn/SSI-ssi-securities-corporation.htm" xr:uid="{3AFCB51F-ADE3-45E8-9A65-60756CA624F4}"/>
-    <hyperlink ref="B14" r:id="rId12" display="https://finance.vietstock.vn/SSB-southeast-asia-commercial-joint-stock-bank.htm" xr:uid="{5F3C9FB2-A4A9-4EDC-BDD8-D23339ADFE21}"/>
-    <hyperlink ref="B15" r:id="rId13" display="https://finance.vietstock.vn/BID-joint-stock-commercial-bank-for-investment-and-development-of-vietnam.htm" xr:uid="{C181908F-AC5D-45AF-9357-F7F3966EBF69}"/>
-    <hyperlink ref="B16" r:id="rId14" display="https://finance.vietstock.vn/SAB-saigon-beer-alcohol-beverage-corporation.htm" xr:uid="{8AB594B4-9FCF-4947-85EE-5666B42F94A4}"/>
-    <hyperlink ref="B17" r:id="rId15" display="https://finance.vietstock.vn/VIB-vietnam-international-commercial-joint-stock-bank.htm" xr:uid="{57F448E0-49A6-46F1-AF4F-C4CAFB75C21E}"/>
-    <hyperlink ref="B18" r:id="rId16" display="https://finance.vietstock.vn/GVR-viet-nam-rubber-group-joint-stock-company.htm" xr:uid="{29DF8571-B0D9-4EDF-8A70-610D76ED3A64}"/>
-    <hyperlink ref="B19" r:id="rId17" display="https://finance.vietstock.vn/LPB-fortune-vietnam-joint-stock-commercial-bank.htm" xr:uid="{D00CF08B-A93C-4BB4-A96D-8827D6E6FFEC}"/>
-    <hyperlink ref="B20" r:id="rId18" display="https://finance.vietstock.vn/CTG-vietnam-joint-stock-commercial-bank-for-industry-and-trade.htm" xr:uid="{7AA361BB-6443-4D81-8539-C320FFF8AF38}"/>
-    <hyperlink ref="B21" r:id="rId19" display="https://finance.vietstock.vn/VCB-joint-stock-commercial-bank-for-foreign-trade-of-vietnam.htm" xr:uid="{1ED1CEA5-0543-40BC-BC46-05CA271EE10D}"/>
-    <hyperlink ref="B22" r:id="rId20" display="https://finance.vietstock.vn/SHB-saigon-hanoi-commercial-joint-stock-bank.htm" xr:uid="{80411AAA-5CF6-48E7-83E2-7B4345D3AEAC}"/>
-    <hyperlink ref="B23" r:id="rId21" display="https://finance.vietstock.vn/TCB-vietnam-technological-and-commercial-joint-stock-bank.htm" xr:uid="{1AF9F40C-F06A-487B-9BE4-640508E5AAEF}"/>
-    <hyperlink ref="B24" r:id="rId22" display="https://finance.vietstock.vn/MBB-military-commercial-joint-stock-bank.htm" xr:uid="{47691AA2-D46E-41FC-AA97-5AD7B372ACFD}"/>
-    <hyperlink ref="B25" r:id="rId23" display="https://finance.vietstock.vn/MWG-mobile-world-investment-corporation.htm" xr:uid="{A0652C5B-4779-4E9D-A1CD-1A036BA525B9}"/>
-    <hyperlink ref="B26" r:id="rId24" display="https://finance.vietstock.vn/VRE-vincom-retail-joint-stock-company.htm" xr:uid="{07B73939-B0AA-4510-B76A-9357E2469803}"/>
-    <hyperlink ref="B27" r:id="rId25" display="https://finance.vietstock.vn/VJC-vietjet-aviation-joint-stock-company.htm" xr:uid="{78AAD0DE-1C7E-43BA-B80D-C96E6E95DFF8}"/>
-    <hyperlink ref="B28" r:id="rId26" display="https://finance.vietstock.vn/HDB-ho-chi-minh-city-development-joint-stock-commercial-bank.htm" xr:uid="{AB438634-E2F8-4DAA-A7E3-9E4174E2B0FF}"/>
-    <hyperlink ref="B29" r:id="rId27" display="https://finance.vietstock.vn/STB-saigon-thuong-tin-commercial-joint-stock-bank.htm" xr:uid="{93075649-2FDB-48D4-B5D6-158853B9F628}"/>
-    <hyperlink ref="B30" r:id="rId28" display="https://finance.vietstock.vn/MSN-masan-group-corporation.htm" xr:uid="{70322973-8ADB-4B30-9FE3-04485D85BAF4}"/>
-    <hyperlink ref="B31" r:id="rId29" display="https://finance.vietstock.vn/VNM-vietnam-dairy-products-joint-stock-company.htm" xr:uid="{06F445D3-067E-4452-9411-E448A1013C8E}"/>
-    <hyperlink ref="B32" r:id="rId30" display="https://finance.vietstock.vn/HPG-hoa-phat-group-joint-stock-company.htm" xr:uid="{B1389BE9-FE91-46DC-AD5D-01D46D27B162}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -4875,14 +4766,14 @@
  +0.16*$E$22
  +0.06*(100-$E$14)
  +0.04*$E$23,0)</f>
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G3" t="s">
         <v>121</v>
       </c>
       <c r="H3">
         <f>Dashboard!E3</f>
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.45">
@@ -4898,7 +4789,7 @@
       </c>
       <c r="E4">
         <f>MAX(0,MIN(100,ROUND(100*(0.35*$B$6+0.25*IFERROR(ABS($B$14)/MAX(ABS($B$11),0.0001),0)+0.2*$B$19+0.2*$B$16-0.15*$B$18-0.05*$B$5),0)))</f>
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="G4" t="s">
         <v>122</v>
@@ -4944,14 +4835,14 @@
       </c>
       <c r="E6">
         <f>MAX(0,MIN(100,ROUND(100*(0.45*$B$5+0.25*$B$18+0.2*(1-$B$19)+0.1*MIN(ABS($B$11)/3,1)-0.2*IFERROR(ABS($B$14)/MAX(ABS($B$11),0.0001),0)),0)))</f>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G6" t="s">
         <v>124</v>
       </c>
       <c r="H6" s="9">
         <f>Dashboard!E13</f>
-        <v>47.338933831376551</v>
+        <v>47.51636141730696</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.45">
@@ -4997,7 +4888,7 @@
       </c>
       <c r="H8" s="9">
         <f>Dashboard!E14</f>
-        <v>57.492227426542783</v>
+        <v>56.736798882994023</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.45">
@@ -5030,7 +4921,7 @@
       </c>
       <c r="H10" s="9">
         <f>Dashboard!E22</f>
-        <v>40</v>
+        <v>36</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.45">
@@ -5039,7 +4930,7 @@
       </c>
       <c r="B11" s="9">
         <f>SUM(AutoScore!T2:T31)</f>
-        <v>-0.26610661686234488</v>
+        <v>-0.24836385826930366</v>
       </c>
       <c r="D11" s="17" t="s">
         <v>123</v>
@@ -5062,7 +4953,7 @@
       </c>
       <c r="B12" s="12">
         <f>SUM(AutoScore!U2:U31)</f>
-        <v>0.35134739481689642</v>
+        <v>0.3190665819201316</v>
       </c>
       <c r="D12" s="17" t="s">
         <v>174</v>
@@ -5085,14 +4976,14 @@
       </c>
       <c r="B13" s="9">
         <f>SUMPRODUCT(AutoScore!T2:T31,AutoScore!K2:K31)</f>
-        <v>-0.29512718158903495</v>
+        <v>-0.26801172415241398</v>
       </c>
       <c r="D13" s="17" t="s">
         <v>175</v>
       </c>
       <c r="E13" s="12">
         <f>MAX(0,MIN(100, 50 + 10*B11))</f>
-        <v>47.338933831376551</v>
+        <v>47.51636141730696</v>
       </c>
       <c r="G13" t="s">
         <v>137</v>
@@ -5110,14 +5001,14 @@
       </c>
       <c r="B14" s="9">
         <f>SUMPRODUCT(AutoScore!T2:T31,AutoScore!L2:L31)</f>
-        <v>0.24155806289596674</v>
+        <v>0.21265801501504911</v>
       </c>
       <c r="D14" s="17" t="s">
         <v>176</v>
       </c>
       <c r="E14" s="12">
         <f>MAX(0,MIN(100, 50 + 10*(B14-B15)))</f>
-        <v>57.492227426542783</v>
+        <v>56.736798882994023</v>
       </c>
       <c r="G14" t="s">
         <v>131</v>
@@ -5135,7 +5026,7 @@
       </c>
       <c r="B15" s="12" cm="1">
         <f t="array" ref="B15">SUMPRODUCT((AutoScore!L2:L31=0)*AutoScore!T2:T31)</f>
-        <v>-0.50766467975831153</v>
+        <v>-0.46102187328435285</v>
       </c>
       <c r="D15" s="17" t="s">
         <v>177</v>
@@ -5158,7 +5049,7 @@
       </c>
       <c r="B16" s="9">
         <f>IFERROR(SUMPRODUCT(AutoScore!T2:T31,AutoScore!K2:K31)/SUM(AutoScore!T2:T31),0)</f>
-        <v>1.1090561560207359</v>
+        <v>1.0791091989793697</v>
       </c>
       <c r="D16" s="17" t="s">
         <v>178</v>
@@ -5181,7 +5072,7 @@
       </c>
       <c r="B17" s="9">
         <f>IFERROR(SUMPRODUCT(AutoScore!T2:T31,AutoScore!L2:L31)/SUM(AutoScore!T2:T31),0)</f>
-        <v>-0.90774917867195715</v>
+        <v>-0.85623575224242843</v>
       </c>
       <c r="D17" s="17" t="s">
         <v>179</v>
@@ -5253,7 +5144,7 @@
       </c>
       <c r="E20" s="10" t="str">
         <f>IF($E$3-$E$15&gt;=MAX(4,MIN(8,ROUND($E$13/15,0))),"Internal&gt;Surface(Bull ẩn)",IF($E$3-$E$15&lt;=-MAX(4,MIN(8,ROUND($E$13/15,0))),"Surface&gt;Internals(Kéo trụ/méo)","ALIGNED"))</f>
-        <v>Internal&gt;Surface(Bull ẩn)</v>
+        <v>ALIGNED</v>
       </c>
       <c r="G20" t="s">
         <v>133</v>
@@ -5295,14 +5186,14 @@
       </c>
       <c r="B22" s="15" t="str">
         <f>TEXT(B14,"0.00")&amp;" / "&amp;TEXT(B15,"0.00")</f>
-        <v>0.24 / -0.51</v>
+        <v>0.21 / -0.46</v>
       </c>
       <c r="D22" s="17" t="s">
         <v>184</v>
       </c>
       <c r="E22">
         <f>MAX(0,MIN(100,ROUND(100*$B$24,0)))</f>
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="G22" t="s">
         <v>135</v>
@@ -5341,7 +5232,7 @@
       </c>
       <c r="B24" s="9">
         <f>IFERROR(SUMIF(AutoScore!$G$2:$G$31,"&gt;0",AutoScore!$J$2:$J$31),0)</f>
-        <v>0.39972426278285372</v>
+        <v>0.36299871898334685</v>
       </c>
       <c r="D24" s="31"/>
       <c r="G24" t="s">
@@ -5358,7 +5249,7 @@
       </c>
       <c r="B25" s="9">
         <f>IFERROR(SUMIF(AutoScore!$G$2:$G$31,"&lt;0",AutoScore!$J$2:$J$31),0)</f>
-        <v>0.57899750140676653</v>
+        <v>0.52580083541086053</v>
       </c>
       <c r="G25" t="s">
         <v>141</v>
@@ -5419,7 +5310,7 @@
 "SCALP (range / intraday only)",
 "WAIT / OBSERVE"
 ))))))</f>
-        <v>WAIT / OBSERVE</v>
+        <v>PULLBACK SHORT (sell LH / EMA reject)</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.45">
@@ -5562,7 +5453,7 @@
         <f t="array" ref="M2">IFERROR(tblOI[[#This Row],[Open interest (OI)]]-INDEX(tblOI[Open interest (OI)],tblOI[[#This Row],[No.]]+1),"")</f>
         <v>6868</v>
       </c>
-      <c r="N2" s="47" t="str">
+      <c r="N2" s="41" t="str">
         <f>IF(OR(tblOI[[#This Row],[ΔClose]]="",tblOI[[#This Row],[ΔOI]]=""),"",
  IF(AND(tblOI[[#This Row],[ΔClose]]&gt;0,tblOI[[#This Row],[ΔOI]]&gt;0),"BUILD LONG",
  IF(AND(tblOI[[#This Row],[ΔClose]]&lt;0,tblOI[[#This Row],[ΔOI]]&gt;0),"BUILD SHORT",
@@ -5570,7 +5461,7 @@
  IF(AND(tblOI[[#This Row],[ΔClose]]&lt;0,tblOI[[#This Row],[ΔOI]]&lt;0),"LONG UNWIND","-")))))</f>
         <v>BUILD LONG</v>
       </c>
-      <c r="O2" s="47">
+      <c r="O2" s="41">
         <f>IF(tblOI[[#This Row],[OI_Quadrant]]="","",1)</f>
         <v>1</v>
       </c>
@@ -5622,7 +5513,7 @@
         <f t="array" ref="M3">IFERROR(tblOI[[#This Row],[Open interest (OI)]]-INDEX(tblOI[Open interest (OI)],tblOI[[#This Row],[No.]]+1),"")</f>
         <v>-5186</v>
       </c>
-      <c r="N3" s="47" t="str">
+      <c r="N3" s="41" t="str">
         <f>IF(OR(tblOI[[#This Row],[ΔClose]]="",tblOI[[#This Row],[ΔOI]]=""),"",
  IF(AND(tblOI[[#This Row],[ΔClose]]&gt;0,tblOI[[#This Row],[ΔOI]]&gt;0),"BUILD LONG",
  IF(AND(tblOI[[#This Row],[ΔClose]]&lt;0,tblOI[[#This Row],[ΔOI]]&gt;0),"BUILD SHORT",
@@ -5630,7 +5521,7 @@
  IF(AND(tblOI[[#This Row],[ΔClose]]&lt;0,tblOI[[#This Row],[ΔOI]]&lt;0),"LONG UNWIND","-")))))</f>
         <v>SHORT COVER</v>
       </c>
-      <c r="O3" s="47">
+      <c r="O3" s="41">
         <f>IF(tblOI[[#This Row],[OI_Quadrant]]="","",1)</f>
         <v>1</v>
       </c>
@@ -6608,15 +6499,15 @@
     <row r="13" spans="1:26" x14ac:dyDescent="0.45">
       <c r="A13" s="23">
         <f ca="1">TODAY()</f>
-        <v>46080</v>
+        <v>46082</v>
       </c>
       <c r="B13" s="46">
         <f ca="1">TIME(HOUR(NOW()), MINUTE(NOW()), SECOND(NOW()))</f>
-        <v>0.64584490740740741</v>
+        <v>0.57420138888888894</v>
       </c>
       <c r="C13" s="20">
         <f>Dashboard!$E$3</f>
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D13" s="21" t="str">
         <f>Dashboard!$B$23</f>
@@ -6656,23 +6547,23 @@
       </c>
       <c r="M13" s="28">
         <f>Dashboard!B11</f>
-        <v>-0.26610661686234488</v>
+        <v>-0.24836385826930366</v>
       </c>
       <c r="N13" s="28">
         <f>Dashboard!E13</f>
-        <v>47.338933831376551</v>
+        <v>47.51636141730696</v>
       </c>
       <c r="O13" s="28">
         <f>Dashboard!E14</f>
-        <v>57.492227426542783</v>
+        <v>56.736798882994023</v>
       </c>
       <c r="P13" s="28">
         <f>Dashboard!B16</f>
-        <v>1.1090561560207359</v>
+        <v>1.0791091989793697</v>
       </c>
       <c r="Q13" s="28">
         <f>Dashboard!B17</f>
-        <v>-0.90774917867195715</v>
+        <v>-0.85623575224242843</v>
       </c>
       <c r="R13" s="20" t="str">
         <f>Dashboard!E17</f>
@@ -6684,19 +6575,19 @@
       </c>
       <c r="T13" s="20">
         <f>Dashboard!E6</f>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="U13" s="28">
         <f>Dashboard!B13</f>
-        <v>-0.29512718158903495</v>
+        <v>-0.26801172415241398</v>
       </c>
       <c r="V13" s="28">
         <f>Dashboard!B14</f>
-        <v>0.24155806289596674</v>
+        <v>0.21265801501504911</v>
       </c>
       <c r="W13" s="28">
         <f>Dashboard!B15</f>
-        <v>-0.50766467975831153</v>
+        <v>-0.46102187328435285</v>
       </c>
       <c r="X13" s="20">
         <f>IF($A14="","",$M14)</f>
@@ -9378,9 +9269,9 @@
       </c>
       <c r="J2">
         <f>IFERROR(
-  _xlfn.XLOOKUP(A2,Raw_VN30_Influence!$B$2:$B$31,Raw_VN30_Influence!$G$2:$G$31)
+  _xlfn.XLOOKUP(A2,Raw_VN30_Influence!$B$2:$B$30,Raw_VN30_Influence!$G$2:$G$30)
   /SUM(Raw_VN30_Influence!$G$2:$G$31),"")</f>
-        <v>4.0370615486432844E-2</v>
+        <v>3.6661476599195802E-2</v>
       </c>
       <c r="K2">
         <f>IF(COUNTIF(Settings!$A:$A,A2)&gt;0,1,0)</f>
@@ -9420,11 +9311,11 @@
       </c>
       <c r="T2" s="8">
         <f>(IF(J2&lt;&gt;"",J2,IF(Raw_VN30_Statistic!R2="",0,Raw_VN30_Statistic!R2/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*G2</f>
-        <v>1.6551952349437463E-2</v>
+        <v>1.5031205405670277E-2</v>
       </c>
       <c r="U2" s="8">
         <f>(IF(J2&lt;&gt;"",J2,IF(Raw_VN30_Statistic!R2="",0,Raw_VN30_Statistic!R2/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*M2</f>
-        <v>3.5324288550628691E-2</v>
+        <v>3.2078792024296289E-2</v>
       </c>
       <c r="V2">
         <f>IFERROR(_xlfn.XLOOKUP(A2,[1]Raw_VN30_Influence!$B$2:$B$31,[1]Raw_VN30_Influence!$I$2:$I$31),"")</f>
@@ -9478,9 +9369,9 @@
       </c>
       <c r="J3">
         <f>IFERROR(
-  _xlfn.XLOOKUP(A3,Raw_VN30_Influence!$B$2:$B$31,Raw_VN30_Influence!$G$2:$G$31)
+  _xlfn.XLOOKUP(A3,Raw_VN30_Influence!$B$2:$B$30,Raw_VN30_Influence!$G$2:$G$30)
   /SUM(Raw_VN30_Influence!$G$2:$G$31),"")</f>
-        <v>5.066561246367461E-3</v>
+        <v>4.6010598137775803E-3</v>
       </c>
       <c r="K3">
         <f>IF(COUNTIF(Settings!$A:$A,A3)&gt;0,1,0)</f>
@@ -9520,11 +9411,11 @@
       </c>
       <c r="T3" s="8">
         <f>(IF(J3&lt;&gt;"",J3,IF(Raw_VN30_Statistic!R3="",0,Raw_VN30_Statistic!R3/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*G3</f>
-        <v>-5.7758798208589054E-3</v>
+        <v>-5.245208187706441E-3</v>
       </c>
       <c r="U3" s="8">
         <f>(IF(J3&lt;&gt;"",J3,IF(Raw_VN30_Statistic!R3="",0,Raw_VN30_Statistic!R3/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*M3</f>
-        <v>1.2666403115918596E-3</v>
+        <v>1.1502649534443899E-3</v>
       </c>
       <c r="V3">
         <f>IFERROR(_xlfn.XLOOKUP(A3,[1]Raw_VN30_Influence!$B$2:$B$31,[1]Raw_VN30_Influence!$I$2:$I$31),"")</f>
@@ -9578,9 +9469,9 @@
       </c>
       <c r="J4">
         <f>IFERROR(
-  _xlfn.XLOOKUP(A4,Raw_VN30_Influence!$B$2:$B$31,Raw_VN30_Influence!$G$2:$G$31)
+  _xlfn.XLOOKUP(A4,Raw_VN30_Influence!$B$2:$B$30,Raw_VN30_Influence!$G$2:$G$30)
   /SUM(Raw_VN30_Influence!$G$2:$G$31),"")</f>
-        <v>1.6783190601148985E-2</v>
+        <v>1.5241198135575767E-2</v>
       </c>
       <c r="K4">
         <f>IF(COUNTIF(Settings!$A:$A,A4)&gt;0,1,0)</f>
@@ -9620,11 +9511,11 @@
       </c>
       <c r="T4" s="8">
         <f>(IF(J4&lt;&gt;"",J4,IF(Raw_VN30_Statistic!R4="",0,Raw_VN30_Statistic!R4/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*G4</f>
-        <v>-1.0909073890746841E-2</v>
+        <v>-9.9067787881242479E-3</v>
       </c>
       <c r="U4" s="8">
         <f>(IF(J4&lt;&gt;"",J4,IF(Raw_VN30_Statistic!R4="",0,Raw_VN30_Statistic!R4/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*M4</f>
-        <v>8.3915953005744923E-3</v>
+        <v>7.6205990677878834E-3</v>
       </c>
       <c r="V4">
         <f>IFERROR(_xlfn.XLOOKUP(A4,[1]Raw_VN30_Influence!$B$2:$B$31,[1]Raw_VN30_Influence!$I$2:$I$31),"")</f>
@@ -9678,9 +9569,9 @@
       </c>
       <c r="J5">
         <f>IFERROR(
-  _xlfn.XLOOKUP(A5,Raw_VN30_Influence!$B$2:$B$31,Raw_VN30_Influence!$G$2:$G$31)
+  _xlfn.XLOOKUP(A5,Raw_VN30_Influence!$B$2:$B$30,Raw_VN30_Influence!$G$2:$G$30)
   /SUM(Raw_VN30_Influence!$G$2:$G$31),"")</f>
-        <v>1.3993884007571766E-2</v>
+        <v>1.2708165206147683E-2</v>
       </c>
       <c r="K5">
         <f>IF(COUNTIF(Settings!$A:$A,A5)&gt;0,1,0)</f>
@@ -9720,11 +9611,11 @@
       </c>
       <c r="T5" s="8">
         <f>(IF(J5&lt;&gt;"",J5,IF(Raw_VN30_Statistic!R5="",0,Raw_VN30_Statistic!R5/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*G5</f>
-        <v>3.7783486820443771E-3</v>
+        <v>3.4312046056598744E-3</v>
       </c>
       <c r="U5" s="8">
         <f>(IF(J5&lt;&gt;"",J5,IF(Raw_VN30_Statistic!R5="",0,Raw_VN30_Statistic!R5/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*M5</f>
-        <v>1.0075596485451655E-2</v>
+        <v>9.1498789484263168E-3</v>
       </c>
       <c r="V5">
         <f>IFERROR(_xlfn.XLOOKUP(A5,[1]Raw_VN30_Influence!$B$2:$B$31,[1]Raw_VN30_Influence!$I$2:$I$31),"")</f>
@@ -9778,9 +9669,9 @@
       </c>
       <c r="J6">
         <f>IFERROR(
-  _xlfn.XLOOKUP(A6,Raw_VN30_Influence!$B$2:$B$31,Raw_VN30_Influence!$G$2:$G$31)
+  _xlfn.XLOOKUP(A6,Raw_VN30_Influence!$B$2:$B$30,Raw_VN30_Influence!$G$2:$G$30)
   /SUM(Raw_VN30_Influence!$G$2:$G$31),"")</f>
-        <v>9.8797393710680775E-2</v>
+        <v>8.9720166362162734E-2</v>
       </c>
       <c r="K6">
         <f>IF(COUNTIF(Settings!$A:$A,A6)&gt;0,1,0)</f>
@@ -9820,11 +9711,11 @@
       </c>
       <c r="T6" s="8">
         <f>(IF(J6&lt;&gt;"",J6,IF(Raw_VN30_Statistic!R6="",0,Raw_VN30_Statistic!R6/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*G6</f>
-        <v>0.26181309333330405</v>
+        <v>0.23775844085973125</v>
       </c>
       <c r="U6" s="8">
         <f>(IF(J6&lt;&gt;"",J6,IF(Raw_VN30_Statistic!R6="",0,Raw_VN30_Statistic!R6/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*M6</f>
-        <v>8.0272882389928329E-2</v>
+        <v>7.2897635169257402E-2</v>
       </c>
       <c r="V6">
         <f>IFERROR(_xlfn.XLOOKUP(A6,[1]Raw_VN30_Influence!$B$2:$B$31,[1]Raw_VN30_Influence!$I$2:$I$31),"")</f>
@@ -9878,9 +9769,9 @@
       </c>
       <c r="J7">
         <f>IFERROR(
-  _xlfn.XLOOKUP(A7,Raw_VN30_Influence!$B$2:$B$31,Raw_VN30_Influence!$G$2:$G$31)
+  _xlfn.XLOOKUP(A7,Raw_VN30_Influence!$B$2:$B$30,Raw_VN30_Influence!$G$2:$G$30)
   /SUM(Raw_VN30_Influence!$G$2:$G$31),"")</f>
-        <v>1.0832376218325737E-2</v>
+        <v>9.8371278826624772E-3</v>
       </c>
       <c r="K7">
         <f>IF(COUNTIF(Settings!$A:$A,A7)&gt;0,1,0)</f>
@@ -9920,11 +9811,11 @@
       </c>
       <c r="T7" s="8">
         <f>(IF(J7&lt;&gt;"",J7,IF(Raw_VN30_Statistic!R7="",0,Raw_VN30_Statistic!R7/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*G7</f>
-        <v>1.9389953430803068E-2</v>
+        <v>1.7608458909965836E-2</v>
       </c>
       <c r="U7" s="8">
         <f>(IF(J7&lt;&gt;"",J7,IF(Raw_VN30_Statistic!R7="",0,Raw_VN30_Statistic!R7/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*M7</f>
-        <v>4.0621410818721575E-3</v>
+        <v>3.6889229559984344E-3</v>
       </c>
       <c r="V7">
         <f>IFERROR(_xlfn.XLOOKUP(A7,[1]Raw_VN30_Influence!$B$2:$B$31,[1]Raw_VN30_Influence!$I$2:$I$31),"")</f>
@@ -9978,9 +9869,9 @@
       </c>
       <c r="J8">
         <f>IFERROR(
-  _xlfn.XLOOKUP(A8,Raw_VN30_Influence!$B$2:$B$31,Raw_VN30_Influence!$G$2:$G$31)
+  _xlfn.XLOOKUP(A8,Raw_VN30_Influence!$B$2:$B$30,Raw_VN30_Influence!$G$2:$G$30)
   /SUM(Raw_VN30_Influence!$G$2:$G$31),"")</f>
-        <v>5.3253401841845344E-3</v>
+        <v>4.8360628688172954E-3</v>
       </c>
       <c r="K8">
         <f>IF(COUNTIF(Settings!$A:$A,A8)&gt;0,1,0)</f>
@@ -10020,11 +9911,11 @@
       </c>
       <c r="T8" s="8">
         <f>(IF(J8&lt;&gt;"",J8,IF(Raw_VN30_Statistic!R8="",0,Raw_VN30_Statistic!R8/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*G8</f>
-        <v>-1.0437666761001687E-2</v>
+        <v>-9.4786832228818986E-3</v>
       </c>
       <c r="U8" s="8">
         <f>(IF(J8&lt;&gt;"",J8,IF(Raw_VN30_Statistic!R8="",0,Raw_VN30_Statistic!R8/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*M8</f>
-        <v>4.260272147347688E-4</v>
+        <v>3.8688502950538913E-4</v>
       </c>
       <c r="V8">
         <f>IFERROR(_xlfn.XLOOKUP(A8,[1]Raw_VN30_Influence!$B$2:$B$31,[1]Raw_VN30_Influence!$I$2:$I$31),"")</f>
@@ -10078,9 +9969,9 @@
       </c>
       <c r="J9">
         <f>IFERROR(
-  _xlfn.XLOOKUP(A9,Raw_VN30_Influence!$B$2:$B$31,Raw_VN30_Influence!$G$2:$G$31)
+  _xlfn.XLOOKUP(A9,Raw_VN30_Influence!$B$2:$B$30,Raw_VN30_Influence!$G$2:$G$30)
   /SUM(Raw_VN30_Influence!$G$2:$G$31),"")</f>
-        <v>4.2151234816008187E-2</v>
+        <v>3.8278497620469074E-2</v>
       </c>
       <c r="K9">
         <f>IF(COUNTIF(Settings!$A:$A,A9)&gt;0,1,0)</f>
@@ -10120,7 +10011,7 @@
       </c>
       <c r="T9" s="8">
         <f>(IF(J9&lt;&gt;"",J9,IF(Raw_VN30_Statistic!R9="",0,Raw_VN30_Statistic!R9/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*G9</f>
-        <v>-6.6598951009292945E-2</v>
+        <v>-6.0480026240341142E-2</v>
       </c>
       <c r="U9" s="8">
         <f>(IF(J9&lt;&gt;"",J9,IF(Raw_VN30_Statistic!R9="",0,Raw_VN30_Statistic!R9/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*M9</f>
@@ -10178,7 +10069,7 @@
       </c>
       <c r="J10" t="str">
         <f>IFERROR(
-  _xlfn.XLOOKUP(A10,Raw_VN30_Influence!$B$2:$B$31,Raw_VN30_Influence!$G$2:$G$31)
+  _xlfn.XLOOKUP(A10,Raw_VN30_Influence!$B$2:$B$30,Raw_VN30_Influence!$G$2:$G$30)
   /SUM(Raw_VN30_Influence!$G$2:$G$31),"")</f>
         <v/>
       </c>
@@ -10278,9 +10169,9 @@
       </c>
       <c r="J11">
         <f>IFERROR(
-  _xlfn.XLOOKUP(A11,Raw_VN30_Influence!$B$2:$B$31,Raw_VN30_Influence!$G$2:$G$31)
+  _xlfn.XLOOKUP(A11,Raw_VN30_Influence!$B$2:$B$30,Raw_VN30_Influence!$G$2:$G$30)
   /SUM(Raw_VN30_Influence!$G$2:$G$31),"")</f>
-        <v>4.6013097517814468E-2</v>
+        <v>4.1785543212061765E-2</v>
       </c>
       <c r="K11">
         <f>IF(COUNTIF(Settings!$A:$A,A11)&gt;0,1,0)</f>
@@ -10320,11 +10211,11 @@
       </c>
       <c r="T11" s="8">
         <f>(IF(J11&lt;&gt;"",J11,IF(Raw_VN30_Statistic!R11="",0,Raw_VN30_Statistic!R11/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*G11</f>
-        <v>-1.0583012429097328E-2</v>
+        <v>-9.6106749387742073E-3</v>
       </c>
       <c r="U11" s="8">
         <f>(IF(J11&lt;&gt;"",J11,IF(Raw_VN30_Statistic!R11="",0,Raw_VN30_Statistic!R11/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*M11</f>
-        <v>8.9057608098995072E-3</v>
+        <v>8.0875244926570545E-3</v>
       </c>
       <c r="V11">
         <f>IFERROR(_xlfn.XLOOKUP(A11,[1]Raw_VN30_Influence!$B$2:$B$31,[1]Raw_VN30_Influence!$I$2:$I$31),"")</f>
@@ -10378,9 +10269,9 @@
       </c>
       <c r="J12">
         <f>IFERROR(
-  _xlfn.XLOOKUP(A12,Raw_VN30_Influence!$B$2:$B$31,Raw_VN30_Influence!$G$2:$G$31)
+  _xlfn.XLOOKUP(A12,Raw_VN30_Influence!$B$2:$B$30,Raw_VN30_Influence!$G$2:$G$30)
   /SUM(Raw_VN30_Influence!$G$2:$G$31),"")</f>
-        <v>4.3230398046053858E-2</v>
+        <v>3.9258510360634699E-2</v>
       </c>
       <c r="K12">
         <f>IF(COUNTIF(Settings!$A:$A,A12)&gt;0,1,0)</f>
@@ -10420,7 +10311,7 @@
       </c>
       <c r="T12" s="8">
         <f>(IF(J12&lt;&gt;"",J12,IF(Raw_VN30_Statistic!R12="",0,Raw_VN30_Statistic!R12/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*G12</f>
-        <v>-4.4959613967896016E-2</v>
+        <v>-4.0828850775060085E-2</v>
       </c>
       <c r="U12" s="8">
         <f>(IF(J12&lt;&gt;"",J12,IF(Raw_VN30_Statistic!R12="",0,Raw_VN30_Statistic!R12/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*M12</f>
@@ -10478,9 +10369,9 @@
       </c>
       <c r="J13">
         <f>IFERROR(
-  _xlfn.XLOOKUP(A13,Raw_VN30_Influence!$B$2:$B$31,Raw_VN30_Influence!$G$2:$G$31)
+  _xlfn.XLOOKUP(A13,Raw_VN30_Influence!$B$2:$B$30,Raw_VN30_Influence!$G$2:$G$30)
   /SUM(Raw_VN30_Influence!$G$2:$G$31),"")</f>
-        <v>5.7032675520944043E-2</v>
+        <v>5.1792673304752977E-2</v>
       </c>
       <c r="K13">
         <f>IF(COUNTIF(Settings!$A:$A,A13)&gt;0,1,0)</f>
@@ -10520,7 +10411,7 @@
       </c>
       <c r="T13" s="8">
         <f>(IF(J13&lt;&gt;"",J13,IF(Raw_VN30_Statistic!R13="",0,Raw_VN30_Statistic!R13/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*G13</f>
-        <v>-9.9236855406442628E-2</v>
+        <v>-9.0119251550270174E-2</v>
       </c>
       <c r="U13" s="8">
         <f>(IF(J13&lt;&gt;"",J13,IF(Raw_VN30_Statistic!R13="",0,Raw_VN30_Statistic!R13/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*M13</f>
@@ -10578,9 +10469,9 @@
       </c>
       <c r="J14">
         <f>IFERROR(
-  _xlfn.XLOOKUP(A14,Raw_VN30_Influence!$B$2:$B$31,Raw_VN30_Influence!$G$2:$G$31)
+  _xlfn.XLOOKUP(A14,Raw_VN30_Influence!$B$2:$B$30,Raw_VN30_Influence!$G$2:$G$30)
   /SUM(Raw_VN30_Influence!$G$2:$G$31),"")</f>
-        <v>8.5324371139651467E-2</v>
+        <v>7.7485007305094986E-2</v>
       </c>
       <c r="K14">
         <f>IF(COUNTIF(Settings!$A:$A,A14)&gt;0,1,0)</f>
@@ -10620,11 +10511,11 @@
       </c>
       <c r="T14" s="8">
         <f>(IF(J14&lt;&gt;"",J14,IF(Raw_VN30_Statistic!R14="",0,Raw_VN30_Statistic!R14/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*G14</f>
-        <v>-4.5221916704015278E-2</v>
+        <v>-4.1067053871700343E-2</v>
       </c>
       <c r="U14" s="8">
         <f>(IF(J14&lt;&gt;"",J14,IF(Raw_VN30_Statistic!R14="",0,Raw_VN30_Statistic!R14/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*M14</f>
-        <v>3.2817065822942582E-2</v>
+        <v>2.9801925886574734E-2</v>
       </c>
       <c r="V14">
         <f>IFERROR(_xlfn.XLOOKUP(A14,[1]Raw_VN30_Influence!$B$2:$B$31,[1]Raw_VN30_Influence!$I$2:$I$31),"")</f>
@@ -10678,9 +10569,9 @@
       </c>
       <c r="J15">
         <f>IFERROR(
-  _xlfn.XLOOKUP(A15,Raw_VN30_Influence!$B$2:$B$31,Raw_VN30_Influence!$G$2:$G$31)
+  _xlfn.XLOOKUP(A15,Raw_VN30_Influence!$B$2:$B$30,Raw_VN30_Influence!$G$2:$G$30)
   /SUM(Raw_VN30_Influence!$G$2:$G$31),"")</f>
-        <v>6.1104864933912281E-3</v>
+        <v>5.5490721379377944E-3</v>
       </c>
       <c r="K15">
         <f>IF(COUNTIF(Settings!$A:$A,A15)&gt;0,1,0)</f>
@@ -10720,11 +10611,11 @@
       </c>
       <c r="T15" s="8">
         <f>(IF(J15&lt;&gt;"",J15,IF(Raw_VN30_Statistic!R15="",0,Raw_VN30_Statistic!R15/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*G15</f>
-        <v>3.1774529765634385E-3</v>
+        <v>2.8855175117276531E-3</v>
       </c>
       <c r="U15" s="8">
         <f>(IF(J15&lt;&gt;"",J15,IF(Raw_VN30_Statistic!R15="",0,Raw_VN30_Statistic!R15/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*M15</f>
-        <v>4.9544485081549992E-4</v>
+        <v>4.4992476794089765E-4</v>
       </c>
       <c r="V15">
         <f>IFERROR(_xlfn.XLOOKUP(A15,[1]Raw_VN30_Influence!$B$2:$B$31,[1]Raw_VN30_Influence!$I$2:$I$31),"")</f>
@@ -10778,9 +10669,9 @@
       </c>
       <c r="J16">
         <f>IFERROR(
-  _xlfn.XLOOKUP(A16,Raw_VN30_Influence!$B$2:$B$31,Raw_VN30_Influence!$G$2:$G$31)
+  _xlfn.XLOOKUP(A16,Raw_VN30_Influence!$B$2:$B$30,Raw_VN30_Influence!$G$2:$G$30)
   /SUM(Raw_VN30_Influence!$G$2:$G$31),"")</f>
-        <v>5.6821247622812652E-3</v>
+        <v>5.1600670808720529E-3</v>
       </c>
       <c r="K16">
         <f>IF(COUNTIF(Settings!$A:$A,A16)&gt;0,1,0)</f>
@@ -10820,11 +10711,11 @@
       </c>
       <c r="T16" s="8">
         <f>(IF(J16&lt;&gt;"",J16,IF(Raw_VN30_Statistic!R16="",0,Raw_VN30_Statistic!R16/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*G16</f>
-        <v>-8.1254384100622086E-3</v>
+        <v>-7.3788959256470355E-3</v>
       </c>
       <c r="U16" s="8">
         <f>(IF(J16&lt;&gt;"",J16,IF(Raw_VN30_Statistic!R16="",0,Raw_VN30_Statistic!R16/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*M16</f>
-        <v>3.3424263307534898E-4</v>
+        <v>3.0353335769833827E-4</v>
       </c>
       <c r="V16">
         <f>IFERROR(_xlfn.XLOOKUP(A16,[1]Raw_VN30_Influence!$B$2:$B$31,[1]Raw_VN30_Influence!$I$2:$I$31),"")</f>
@@ -10878,9 +10769,9 @@
       </c>
       <c r="J17">
         <f>IFERROR(
-  _xlfn.XLOOKUP(A17,Raw_VN30_Influence!$B$2:$B$31,Raw_VN30_Influence!$G$2:$G$31)
+  _xlfn.XLOOKUP(A17,Raw_VN30_Influence!$B$2:$B$30,Raw_VN30_Influence!$G$2:$G$30)
   /SUM(Raw_VN30_Influence!$G$2:$G$31),"")</f>
-        <v>2.0696809090518676E-2</v>
+        <v>1.8795244338176403E-2</v>
       </c>
       <c r="K17">
         <f>IF(COUNTIF(Settings!$A:$A,A17)&gt;0,1,0)</f>
@@ -10920,11 +10811,11 @@
       </c>
       <c r="T17" s="8">
         <f>(IF(J17&lt;&gt;"",J17,IF(Raw_VN30_Statistic!R17="",0,Raw_VN30_Statistic!R17/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*G17</f>
-        <v>-2.566404327224316E-2</v>
+        <v>-2.3306102979338741E-2</v>
       </c>
       <c r="U17" s="8">
         <f>(IF(J17&lt;&gt;"",J17,IF(Raw_VN30_Statistic!R17="",0,Raw_VN30_Statistic!R17/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*M17</f>
-        <v>6.8989363635062247E-3</v>
+        <v>6.2650814460588006E-3</v>
       </c>
       <c r="V17">
         <f>IFERROR(_xlfn.XLOOKUP(A17,[1]Raw_VN30_Influence!$B$2:$B$31,[1]Raw_VN30_Influence!$I$2:$I$31),"")</f>
@@ -10978,9 +10869,9 @@
       </c>
       <c r="J18">
         <f>IFERROR(
-  _xlfn.XLOOKUP(A18,Raw_VN30_Influence!$B$2:$B$31,Raw_VN30_Influence!$G$2:$G$31)
+  _xlfn.XLOOKUP(A18,Raw_VN30_Influence!$B$2:$B$30,Raw_VN30_Influence!$G$2:$G$30)
   /SUM(Raw_VN30_Influence!$G$2:$G$31),"")</f>
-        <v>9.0539592626892561E-3</v>
+        <v>8.2221068873895384E-3</v>
       </c>
       <c r="K18">
         <f>IF(COUNTIF(Settings!$A:$A,A18)&gt;0,1,0)</f>
@@ -11020,11 +10911,11 @@
       </c>
       <c r="T18" s="8">
         <f>(IF(J18&lt;&gt;"",J18,IF(Raw_VN30_Statistic!R18="",0,Raw_VN30_Statistic!R18/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*G18</f>
-        <v>-5.3418359649866605E-3</v>
+        <v>-4.8510430635598277E-3</v>
       </c>
       <c r="U18" s="8">
         <f>(IF(J18&lt;&gt;"",J18,IF(Raw_VN30_Statistic!R18="",0,Raw_VN30_Statistic!R18/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*M18</f>
-        <v>5.432375557613502E-3</v>
+        <v>4.9332641324336766E-3</v>
       </c>
       <c r="V18">
         <f>IFERROR(_xlfn.XLOOKUP(A18,[1]Raw_VN30_Influence!$B$2:$B$31,[1]Raw_VN30_Influence!$I$2:$I$31),"")</f>
@@ -11078,9 +10969,9 @@
       </c>
       <c r="J19">
         <f>IFERROR(
-  _xlfn.XLOOKUP(A19,Raw_VN30_Influence!$B$2:$B$31,Raw_VN30_Influence!$G$2:$G$31)
+  _xlfn.XLOOKUP(A19,Raw_VN30_Influence!$B$2:$B$30,Raw_VN30_Influence!$G$2:$G$30)
   /SUM(Raw_VN30_Influence!$G$2:$G$31),"")</f>
-        <v>2.1278235810380016E-2</v>
+        <v>1.9323251202265634E-2</v>
       </c>
       <c r="K19">
         <f>IF(COUNTIF(Settings!$A:$A,A19)&gt;0,1,0)</f>
@@ -11124,7 +11015,7 @@
       </c>
       <c r="U19" s="8">
         <f>(IF(J19&lt;&gt;"",J19,IF(Raw_VN30_Statistic!R19="",0,Raw_VN30_Statistic!R19/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*M19</f>
-        <v>7.5099655801340402E-3</v>
+        <v>6.8199710125642658E-3</v>
       </c>
       <c r="V19">
         <f>IFERROR(_xlfn.XLOOKUP(A19,[1]Raw_VN30_Influence!$B$2:$B$31,[1]Raw_VN30_Influence!$I$2:$I$31),"")</f>
@@ -11178,9 +11069,9 @@
       </c>
       <c r="J20">
         <f>IFERROR(
-  _xlfn.XLOOKUP(A20,Raw_VN30_Influence!$B$2:$B$31,Raw_VN30_Influence!$G$2:$G$31)
+  _xlfn.XLOOKUP(A20,Raw_VN30_Influence!$B$2:$B$30,Raw_VN30_Influence!$G$2:$G$30)
   /SUM(Raw_VN30_Influence!$G$2:$G$31),"")</f>
-        <v>4.4181823587645136E-2</v>
+        <v>4.0122521592780715E-2</v>
       </c>
       <c r="K20">
         <f>IF(COUNTIF(Settings!$A:$A,A20)&gt;0,1,0)</f>
@@ -11220,7 +11111,7 @@
       </c>
       <c r="T20" s="8">
         <f>(IF(J20&lt;&gt;"",J20,IF(Raw_VN30_Statistic!R20="",0,Raw_VN30_Statistic!R20/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*G20</f>
-        <v>-9.8967284836325109E-2</v>
+        <v>-8.9874448367828805E-2</v>
       </c>
       <c r="U20" s="8">
         <f>(IF(J20&lt;&gt;"",J20,IF(Raw_VN30_Statistic!R20="",0,Raw_VN30_Statistic!R20/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*M20</f>
@@ -11278,9 +11169,9 @@
       </c>
       <c r="J21">
         <f>IFERROR(
-  _xlfn.XLOOKUP(A21,Raw_VN30_Influence!$B$2:$B$31,Raw_VN30_Influence!$G$2:$G$31)
+  _xlfn.XLOOKUP(A21,Raw_VN30_Influence!$B$2:$B$30,Raw_VN30_Influence!$G$2:$G$30)
   /SUM(Raw_VN30_Influence!$G$2:$G$31),"")</f>
-        <v>5.3210455550037401E-2</v>
+        <v>4.8321628181166365E-2</v>
       </c>
       <c r="K21">
         <f>IF(COUNTIF(Settings!$A:$A,A21)&gt;0,1,0)</f>
@@ -11320,11 +11211,11 @@
       </c>
       <c r="T21" s="8">
         <f>(IF(J21&lt;&gt;"",J21,IF(Raw_VN30_Statistic!R21="",0,Raw_VN30_Statistic!R21/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*G21</f>
-        <v>-2.9265750552520575E-2</v>
+        <v>-2.6576895499641501E-2</v>
       </c>
       <c r="U21" s="8">
         <f>(IF(J21&lt;&gt;"",J21,IF(Raw_VN30_Statistic!R21="",0,Raw_VN30_Statistic!R21/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*M21</f>
-        <v>3.8698513127299987E-2</v>
+        <v>3.5143002313575596E-2</v>
       </c>
       <c r="V21">
         <f>IFERROR(_xlfn.XLOOKUP(A21,[1]Raw_VN30_Influence!$B$2:$B$31,[1]Raw_VN30_Influence!$I$2:$I$31),"")</f>
@@ -11378,9 +11269,9 @@
       </c>
       <c r="J22">
         <f>IFERROR(
-  _xlfn.XLOOKUP(A22,Raw_VN30_Influence!$B$2:$B$31,Raw_VN30_Influence!$G$2:$G$31)
+  _xlfn.XLOOKUP(A22,Raw_VN30_Influence!$B$2:$B$30,Raw_VN30_Influence!$G$2:$G$30)
   /SUM(Raw_VN30_Influence!$G$2:$G$31),"")</f>
-        <v>1.0572496093539229E-2</v>
+        <v>9.6011248146225924E-3</v>
       </c>
       <c r="K22">
         <f>IF(COUNTIF(Settings!$A:$A,A22)&gt;0,1,0)</f>
@@ -11420,11 +11311,11 @@
       </c>
       <c r="T22" s="8">
         <f>(IF(J22&lt;&gt;"",J22,IF(Raw_VN30_Statistic!R22="",0,Raw_VN30_Statistic!R22/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*G22</f>
-        <v>2.8545739452555921E-3</v>
+        <v>2.5923036999481001E-3</v>
       </c>
       <c r="U22" s="8">
         <f>(IF(J22&lt;&gt;"",J22,IF(Raw_VN30_Statistic!R22="",0,Raw_VN30_Statistic!R22/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*M22</f>
-        <v>3.5241653645130488E-3</v>
+        <v>3.2003749382075054E-3</v>
       </c>
       <c r="V22">
         <f>IFERROR(_xlfn.XLOOKUP(A22,[1]Raw_VN30_Influence!$B$2:$B$31,[1]Raw_VN30_Influence!$I$2:$I$31),"")</f>
@@ -11478,9 +11369,9 @@
       </c>
       <c r="J23">
         <f>IFERROR(
-  _xlfn.XLOOKUP(A23,Raw_VN30_Influence!$B$2:$B$31,Raw_VN30_Influence!$G$2:$G$31)
+  _xlfn.XLOOKUP(A23,Raw_VN30_Influence!$B$2:$B$30,Raw_VN30_Influence!$G$2:$G$30)
   /SUM(Raw_VN30_Influence!$G$2:$G$31),"")</f>
-        <v>2.2466416550399684E-2</v>
+        <v>2.0402265229447988E-2</v>
       </c>
       <c r="K23">
         <f>IF(COUNTIF(Settings!$A:$A,A23)&gt;0,1,0)</f>
@@ -11520,11 +11411,11 @@
       </c>
       <c r="T23" s="8">
         <f>(IF(J23&lt;&gt;"",J23,IF(Raw_VN30_Statistic!R23="",0,Raw_VN30_Statistic!R23/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*G23</f>
-        <v>-1.7074476578303761E-2</v>
+        <v>-1.550572157438047E-2</v>
       </c>
       <c r="U23" s="8">
         <f>(IF(J23&lt;&gt;"",J23,IF(Raw_VN30_Statistic!R23="",0,Raw_VN30_Statistic!R23/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*M23</f>
-        <v>1.4041510344000926E-3</v>
+        <v>1.2751415768406011E-3</v>
       </c>
       <c r="V23">
         <f>IFERROR(_xlfn.XLOOKUP(A23,[1]Raw_VN30_Influence!$B$2:$B$31,[1]Raw_VN30_Influence!$I$2:$I$31),"")</f>
@@ -11578,9 +11469,9 @@
       </c>
       <c r="J24">
         <f>IFERROR(
-  _xlfn.XLOOKUP(A24,Raw_VN30_Influence!$B$2:$B$31,Raw_VN30_Influence!$G$2:$G$31)
+  _xlfn.XLOOKUP(A24,Raw_VN30_Influence!$B$2:$B$30,Raw_VN30_Influence!$G$2:$G$30)
   /SUM(Raw_VN30_Influence!$G$2:$G$31),"")</f>
-        <v>4.1805462107605808E-2</v>
+        <v>3.7964493538416015E-2</v>
       </c>
       <c r="K24">
         <f>IF(COUNTIF(Settings!$A:$A,A24)&gt;0,1,0)</f>
@@ -11620,11 +11511,11 @@
       </c>
       <c r="T24" s="8">
         <f>(IF(J24&lt;&gt;"",J24,IF(Raw_VN30_Statistic!R24="",0,Raw_VN30_Statistic!R24/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*G24</f>
-        <v>1.5468020979814149E-2</v>
+        <v>1.4046862609213926E-2</v>
       </c>
       <c r="U24" s="8">
         <f>(IF(J24&lt;&gt;"",J24,IF(Raw_VN30_Statistic!R24="",0,Raw_VN30_Statistic!R24/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*M24</f>
-        <v>2.9007871666502004E-2</v>
+        <v>2.6342709802166228E-2</v>
       </c>
       <c r="V24">
         <f>IFERROR(_xlfn.XLOOKUP(A24,[1]Raw_VN30_Influence!$B$2:$B$31,[1]Raw_VN30_Influence!$I$2:$I$31),"")</f>
@@ -11678,9 +11569,9 @@
       </c>
       <c r="J25">
         <f>IFERROR(
-  _xlfn.XLOOKUP(A25,Raw_VN30_Influence!$B$2:$B$31,Raw_VN30_Influence!$G$2:$G$31)
+  _xlfn.XLOOKUP(A25,Raw_VN30_Influence!$B$2:$B$30,Raw_VN30_Influence!$G$2:$G$30)
   /SUM(Raw_VN30_Influence!$G$2:$G$31),"")</f>
-        <v>1.4416739803834558E-2</v>
+        <v>1.309217019821258E-2</v>
       </c>
       <c r="K25">
         <f>IF(COUNTIF(Settings!$A:$A,A25)&gt;0,1,0)</f>
@@ -11720,7 +11611,7 @@
       </c>
       <c r="T25" s="8">
         <f>(IF(J25&lt;&gt;"",J25,IF(Raw_VN30_Statistic!R25="",0,Raw_VN30_Statistic!R25/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*G25</f>
-        <v>-8.2175416881856977E-3</v>
+        <v>-7.4625370129811699E-3</v>
       </c>
       <c r="U25" s="8">
         <f>(IF(J25&lt;&gt;"",J25,IF(Raw_VN30_Statistic!R25="",0,Raw_VN30_Statistic!R25/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*M25</f>
@@ -11778,9 +11669,9 @@
       </c>
       <c r="J26">
         <f>IFERROR(
-  _xlfn.XLOOKUP(A26,Raw_VN30_Influence!$B$2:$B$31,Raw_VN30_Influence!$G$2:$G$31)
+  _xlfn.XLOOKUP(A26,Raw_VN30_Influence!$B$2:$B$30,Raw_VN30_Influence!$G$2:$G$30)
   /SUM(Raw_VN30_Influence!$G$2:$G$31),"")</f>
-        <v>0.11828179594785224</v>
+        <v>0.10741439638715307</v>
       </c>
       <c r="K26">
         <f>IF(COUNTIF(Settings!$A:$A,A26)&gt;0,1,0)</f>
@@ -11820,11 +11711,11 @@
       </c>
       <c r="T26" s="8">
         <f>(IF(J26&lt;&gt;"",J26,IF(Raw_VN30_Statistic!R26="",0,Raw_VN30_Statistic!R26/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*G26</f>
-        <v>0.21763850454404812</v>
+        <v>0.19764248935236164</v>
       </c>
       <c r="U26" s="8">
         <f>(IF(J26&lt;&gt;"",J26,IF(Raw_VN30_Statistic!R26="",0,Raw_VN30_Statistic!R26/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*M26</f>
-        <v>4.505973178965799E-2</v>
+        <v>4.0919770052248783E-2</v>
       </c>
       <c r="V26">
         <f>IFERROR(_xlfn.XLOOKUP(A26,[1]Raw_VN30_Influence!$B$2:$B$31,[1]Raw_VN30_Influence!$I$2:$I$31),"")</f>
@@ -11878,9 +11769,9 @@
       </c>
       <c r="J27">
         <f>IFERROR(
-  _xlfn.XLOOKUP(A27,Raw_VN30_Influence!$B$2:$B$31,Raw_VN30_Influence!$G$2:$G$31)
+  _xlfn.XLOOKUP(A27,Raw_VN30_Influence!$B$2:$B$30,Raw_VN30_Influence!$G$2:$G$30)
   /SUM(Raw_VN30_Influence!$G$2:$G$31),"")</f>
-        <v>3.8946780734954223E-2</v>
+        <v>3.5368459789977276E-2</v>
       </c>
       <c r="K27">
         <f>IF(COUNTIF(Settings!$A:$A,A27)&gt;0,1,0)</f>
@@ -11920,11 +11811,11 @@
       </c>
       <c r="T27" s="8">
         <f>(IF(J27&lt;&gt;"",J27,IF(Raw_VN30_Statistic!R27="",0,Raw_VN30_Statistic!R27/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*G27</f>
-        <v>-5.880963890978088E-2</v>
+        <v>-5.3406374282865689E-2</v>
       </c>
       <c r="U27" s="8">
         <f>(IF(J27&lt;&gt;"",J27,IF(Raw_VN30_Statistic!R27="",0,Raw_VN30_Statistic!R27/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*M27</f>
-        <v>7.0812328609010109E-3</v>
+        <v>6.4306290527233623E-3</v>
       </c>
       <c r="V27">
         <f>IFERROR(_xlfn.XLOOKUP(A27,[1]Raw_VN30_Influence!$B$2:$B$31,[1]Raw_VN30_Influence!$I$2:$I$31),"")</f>
@@ -11978,9 +11869,9 @@
       </c>
       <c r="J28">
         <f>IFERROR(
-  _xlfn.XLOOKUP(A28,Raw_VN30_Influence!$B$2:$B$31,Raw_VN30_Influence!$G$2:$G$31)
+  _xlfn.XLOOKUP(A28,Raw_VN30_Influence!$B$2:$B$30,Raw_VN30_Influence!$G$2:$G$30)
   /SUM(Raw_VN30_Influence!$G$2:$G$31),"")</f>
-        <v>4.7443539391109693E-2</v>
+        <v>4.3084560099281299E-2</v>
       </c>
       <c r="K28">
         <f>IF(COUNTIF(Settings!$A:$A,A28)&gt;0,1,0)</f>
@@ -12020,11 +11911,11 @@
       </c>
       <c r="T28" s="8">
         <f>(IF(J28&lt;&gt;"",J28,IF(Raw_VN30_Statistic!R28="",0,Raw_VN30_Statistic!R28/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*G28</f>
-        <v>-0.16130803392977294</v>
+        <v>-0.14648750433755642</v>
       </c>
       <c r="U28" s="8">
         <f>(IF(J28&lt;&gt;"",J28,IF(Raw_VN30_Statistic!R28="",0,Raw_VN30_Statistic!R28/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*M28</f>
-        <v>3.6495030300854213E-3</v>
+        <v>3.3141969307140008E-3</v>
       </c>
       <c r="V28">
         <f>IFERROR(_xlfn.XLOOKUP(A28,[1]Raw_VN30_Influence!$B$2:$B$31,[1]Raw_VN30_Influence!$I$2:$I$31),"")</f>
@@ -12078,9 +11969,9 @@
       </c>
       <c r="J29">
         <f>IFERROR(
-  _xlfn.XLOOKUP(A29,Raw_VN30_Influence!$B$2:$B$31,Raw_VN30_Influence!$G$2:$G$31)
+  _xlfn.XLOOKUP(A29,Raw_VN30_Influence!$B$2:$B$30,Raw_VN30_Influence!$G$2:$G$30)
   /SUM(Raw_VN30_Influence!$G$2:$G$31),"")</f>
-        <v>5.190444780428826E-2</v>
+        <v>4.7135612762965927E-2</v>
       </c>
       <c r="K29">
         <f>IF(COUNTIF(Settings!$A:$A,A29)&gt;0,1,0)</f>
@@ -12120,11 +12011,11 @@
       </c>
       <c r="T29" s="8">
         <f>(IF(J29&lt;&gt;"",J29,IF(Raw_VN30_Statistic!R29="",0,Raw_VN30_Statistic!R29/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*G29</f>
-        <v>8.8237561267290043E-3</v>
+        <v>8.0130541697042076E-3</v>
       </c>
       <c r="U29" s="8">
         <f>(IF(J29&lt;&gt;"",J29,IF(Raw_VN30_Statistic!R29="",0,Raw_VN30_Statistic!R29/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*M29</f>
-        <v>1.4829842229796608E-2</v>
+        <v>1.3467317932275945E-2</v>
       </c>
       <c r="V29">
         <f>IFERROR(_xlfn.XLOOKUP(A29,[1]Raw_VN30_Influence!$B$2:$B$31,[1]Raw_VN30_Influence!$I$2:$I$31),"")</f>
@@ -12178,9 +12069,9 @@
       </c>
       <c r="J30">
         <f>IFERROR(
-  _xlfn.XLOOKUP(A30,Raw_VN30_Influence!$B$2:$B$31,Raw_VN30_Influence!$G$2:$G$31)
+  _xlfn.XLOOKUP(A30,Raw_VN30_Influence!$B$2:$B$30,Raw_VN30_Influence!$G$2:$G$30)
   /SUM(Raw_VN30_Influence!$G$2:$G$31),"")</f>
-        <v>7.055304913165905E-3</v>
+        <v>6.4070832920827998E-3</v>
       </c>
       <c r="K30">
         <f>IF(COUNTIF(Settings!$A:$A,A30)&gt;0,1,0)</f>
@@ -12220,11 +12111,11 @@
       </c>
       <c r="T30" s="8">
         <f>(IF(J30&lt;&gt;"",J30,IF(Raw_VN30_Statistic!R30="",0,Raw_VN30_Statistic!R30/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*G30</f>
-        <v>1.5521670808964992E-2</v>
+        <v>1.4095583242582161E-2</v>
       </c>
       <c r="U30" s="8">
         <f>(IF(J30&lt;&gt;"",J30,IF(Raw_VN30_Statistic!R30="",0,Raw_VN30_Statistic!R30/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*M30</f>
-        <v>5.8794207609715972E-3</v>
+        <v>5.3392360767356749E-3</v>
       </c>
       <c r="V30">
         <f>IFERROR(_xlfn.XLOOKUP(A30,[1]Raw_VN30_Influence!$B$2:$B$31,[1]Raw_VN30_Influence!$I$2:$I$31),"")</f>
@@ -12278,9 +12169,9 @@
       </c>
       <c r="J31">
         <f>IFERROR(
-  _xlfn.XLOOKUP(A31,Raw_VN30_Influence!$B$2:$B$31,Raw_VN30_Influence!$G$2:$G$31)
+  _xlfn.XLOOKUP(A31,Raw_VN30_Influence!$B$2:$B$30,Raw_VN30_Influence!$G$2:$G$30)
   /SUM(Raw_VN30_Influence!$G$2:$G$31),"")</f>
-        <v>2.1971983601123658E-2</v>
+        <v>1.9953259392372108E-2</v>
       </c>
       <c r="K31">
         <f>IF(COUNTIF(Settings!$A:$A,A31)&gt;0,1,0)</f>
@@ -12320,7 +12211,7 @@
       </c>
       <c r="T31" s="8">
         <f>(IF(J31&lt;&gt;"",J31,IF(Raw_VN30_Statistic!R31="",0,Raw_VN30_Statistic!R31/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*G31</f>
-        <v>-5.1634161462640597E-2</v>
+        <v>-4.6890159572074458E-2</v>
       </c>
       <c r="U31" s="8">
         <f>(IF(J31&lt;&gt;"",J31,IF(Raw_VN30_Statistic!R31="",0,Raw_VN30_Statistic!R31/SUM(Raw_VN30_Statistic!$R$2:$R$31))))*M31</f>

</xml_diff>